<commit_message>
Inserção Dados complementares Origem/Desativação temporária CMC
</commit_message>
<xml_diff>
--- a/TemplateAC_ORIGEM.xlsx
+++ b/TemplateAC_ORIGEM.xlsx
@@ -372,7 +372,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -474,6 +474,39 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -973,21 +1006,25 @@
     <row r="6" ht="34.5" customHeight="1" s="14">
       <c r="A6" s="30" t="inlineStr">
         <is>
-          <t>PT-SG-122104-01</t>
+          <t>PDT-SG-122104-01</t>
         </is>
       </c>
       <c r="B6" s="10" t="n"/>
-      <c r="C6" s="40" t="n"/>
+      <c r="C6" s="30" t="inlineStr">
+        <is>
+          <t>PILAR</t>
+        </is>
+      </c>
       <c r="D6" s="9" t="n"/>
       <c r="E6" s="10" t="n"/>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>SAP:</t>
-        </is>
-      </c>
-      <c r="G6" s="37" t="inlineStr">
-        <is>
-          <t>CE: AC-1900.0000-6252-811-O2C-</t>
+      <c r="F6" s="54" t="inlineStr">
+        <is>
+          <t>SAP: 123456778</t>
+        </is>
+      </c>
+      <c r="G6" s="30" t="inlineStr">
+        <is>
+          <t>CE: AC-1900.0000-6252-811-O2C-28</t>
         </is>
       </c>
       <c r="H6" s="10" t="n"/>
@@ -1011,7 +1048,7 @@
       <c r="B8" s="26" t="n"/>
       <c r="C8" s="34" t="inlineStr">
         <is>
-          <t>[ ✔ ] Transmissor de pressão estática (PT)</t>
+          <t>[ ] Transmissor de pressão estática (PT)</t>
         </is>
       </c>
       <c r="D8" s="31" t="n"/>
@@ -1029,7 +1066,7 @@
       <c r="B9" s="18" t="n"/>
       <c r="C9" s="22" t="inlineStr">
         <is>
-          <t>[ ] Transmissor de pressão diferencial (PDT)</t>
+          <t>[ ✔ ] Transmissor de pressão diferencial (PDT)</t>
         </is>
       </c>
       <c r="E9" s="18" t="n"/>
@@ -1075,7 +1112,7 @@
     <row r="13">
       <c r="A13" s="30" t="inlineStr">
         <is>
-          <t>25-ODS-0638 - PRE - 230</t>
+          <t>25-ODS-0638 - PRE - 231</t>
         </is>
       </c>
       <c r="B13" s="9" t="n"/>
@@ -1697,7 +1734,7 @@
       <c r="H43" s="29" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="49" t="inlineStr">
+      <c r="A45" s="60" t="inlineStr">
         <is>
           <t>Data: 12/09/2025</t>
         </is>

</xml_diff>

<commit_message>
Ajuste dados complementares ORIGEM + Desativação CMC + ajuste layout tela consulta bd
</commit_message>
<xml_diff>
--- a/TemplateAC_ORIGEM.xlsx
+++ b/TemplateAC_ORIGEM.xlsx
@@ -372,7 +372,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -501,6 +501,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -1006,7 +1009,7 @@
     <row r="6" ht="34.5" customHeight="1" s="14">
       <c r="A6" s="30" t="inlineStr">
         <is>
-          <t>PDT-SG-122104-01</t>
+          <t>TT-SG-122104-01</t>
         </is>
       </c>
       <c r="B6" s="10" t="n"/>
@@ -1019,12 +1022,12 @@
       <c r="E6" s="10" t="n"/>
       <c r="F6" s="54" t="inlineStr">
         <is>
-          <t>SAP: 123456778</t>
+          <t>SAP: 123456</t>
         </is>
       </c>
       <c r="G6" s="30" t="inlineStr">
         <is>
-          <t>CE: AC-1900.0000-6252-811-O2C-28</t>
+          <t>CE: 8902658</t>
         </is>
       </c>
       <c r="H6" s="10" t="n"/>
@@ -1066,7 +1069,7 @@
       <c r="B9" s="18" t="n"/>
       <c r="C9" s="22" t="inlineStr">
         <is>
-          <t>[ ✔ ] Transmissor de pressão diferencial (PDT)</t>
+          <t>[ ] Transmissor de pressão diferencial (PDT)</t>
         </is>
       </c>
       <c r="E9" s="18" t="n"/>
@@ -1078,7 +1081,7 @@
       <c r="B10" s="29" t="n"/>
       <c r="C10" s="44" t="inlineStr">
         <is>
-          <t>[ ] Transmissor de temperatura (TT)</t>
+          <t>[ ✔ ] Transmissor de temperatura (TT)</t>
         </is>
       </c>
       <c r="D10" s="32" t="n"/>
@@ -1112,7 +1115,7 @@
     <row r="13">
       <c r="A13" s="30" t="inlineStr">
         <is>
-          <t>25-ODS-0638 - PRE - 231</t>
+          <t>25-ODS-0638 - TEM - 150</t>
         </is>
       </c>
       <c r="B13" s="9" t="n"/>
@@ -1714,7 +1717,17 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="30" t="inlineStr"/>
+      <c r="A42" s="30" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t xml:space="preserve">Novo NS alterado no computador de vazão / XML / SFP
+</t>
+          </r>
+        </is>
+      </c>
       <c r="B42" s="31" t="n"/>
       <c r="C42" s="31" t="n"/>
       <c r="D42" s="31" t="n"/>
@@ -1734,7 +1747,7 @@
       <c r="H43" s="29" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="60" t="inlineStr">
+      <c r="A45" s="61" t="inlineStr">
         <is>
           <t>Data: 12/09/2025</t>
         </is>

</xml_diff>

<commit_message>
Ajuste AC Origem centralização de data e Descrição TT+TE
</commit_message>
<xml_diff>
--- a/TemplateAC_ORIGEM.xlsx
+++ b/TemplateAC_ORIGEM.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="13320" yWindow="-16485" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-13380" yWindow="-16320" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Template Formulário" sheetId="1" state="visible" r:id="rId1"/>
@@ -339,6 +339,17 @@
     </border>
     <border>
       <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
       <right/>
       <top style="thin">
         <color rgb="FF000000"/>
@@ -353,17 +364,6 @@
       </right>
       <top style="thin">
         <color rgb="FF000000"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
       </top>
       <bottom/>
       <diagonal/>
@@ -372,7 +372,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -386,136 +386,91 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -930,109 +885,109 @@
   <dimension ref="A1:O49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
-    <col width="15" customWidth="1" style="14" min="1" max="4"/>
-    <col width="11.7265625" customWidth="1" style="14" min="5" max="5"/>
-    <col width="12.453125" customWidth="1" style="14" min="6" max="6"/>
-    <col width="10" customWidth="1" style="14" min="7" max="7"/>
-    <col width="15" customWidth="1" style="14" min="8" max="8"/>
+    <col width="15" customWidth="1" style="15" min="1" max="4"/>
+    <col width="11.7265625" customWidth="1" style="15" min="5" max="5"/>
+    <col width="12.453125" customWidth="1" style="15" min="6" max="6"/>
+    <col width="10" customWidth="1" style="15" min="7" max="7"/>
+    <col width="15" customWidth="1" style="15" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20" customHeight="1" s="14">
-      <c r="A1" s="25" t="n"/>
-      <c r="B1" s="26" t="n"/>
-      <c r="C1" s="43" t="inlineStr">
+    <row r="1" ht="20" customHeight="1" s="15">
+      <c r="A1" s="29" t="n"/>
+      <c r="B1" s="11" t="n"/>
+      <c r="C1" s="12" t="inlineStr">
         <is>
           <t>REGISTRO DE ANÁLISE CRÍTICA DE CERTIFICADO DE CALIBRAÇÃO DE SECUNDÁRIOS</t>
         </is>
       </c>
-      <c r="D1" s="31" t="n"/>
-      <c r="E1" s="31" t="n"/>
-      <c r="F1" s="26" t="n"/>
-      <c r="G1" s="42" t="inlineStr">
+      <c r="D1" s="13" t="n"/>
+      <c r="E1" s="13" t="n"/>
+      <c r="F1" s="11" t="n"/>
+      <c r="G1" s="10" t="inlineStr">
         <is>
           <t>FO-COR-GER-CPROD-030</t>
         </is>
       </c>
-      <c r="H1" s="26" t="n"/>
-    </row>
-    <row r="2" ht="20" customHeight="1" s="14">
-      <c r="A2" s="27" t="n"/>
-      <c r="B2" s="18" t="n"/>
-      <c r="C2" s="27" t="n"/>
-      <c r="F2" s="18" t="n"/>
-      <c r="G2" s="17" t="inlineStr">
+      <c r="H1" s="11" t="n"/>
+    </row>
+    <row r="2" ht="20" customHeight="1" s="15">
+      <c r="A2" s="14" t="n"/>
+      <c r="B2" s="16" t="n"/>
+      <c r="C2" s="14" t="n"/>
+      <c r="F2" s="16" t="n"/>
+      <c r="G2" s="39" t="inlineStr">
         <is>
           <t>Revisão: 0</t>
         </is>
       </c>
-      <c r="H2" s="18" t="n"/>
-    </row>
-    <row r="3" ht="20" customHeight="1" s="14">
-      <c r="A3" s="28" t="n"/>
-      <c r="B3" s="29" t="n"/>
-      <c r="C3" s="28" t="n"/>
-      <c r="D3" s="32" t="n"/>
-      <c r="E3" s="32" t="n"/>
-      <c r="F3" s="29" t="n"/>
-      <c r="G3" s="39" t="inlineStr">
+      <c r="H2" s="16" t="n"/>
+    </row>
+    <row r="3" ht="20" customHeight="1" s="15">
+      <c r="A3" s="17" t="n"/>
+      <c r="B3" s="19" t="n"/>
+      <c r="C3" s="17" t="n"/>
+      <c r="D3" s="18" t="n"/>
+      <c r="E3" s="18" t="n"/>
+      <c r="F3" s="19" t="n"/>
+      <c r="G3" s="38" t="inlineStr">
         <is>
           <t>Página: 1/1</t>
         </is>
       </c>
-      <c r="H3" s="29" t="n"/>
+      <c r="H3" s="19" t="n"/>
     </row>
     <row r="4">
       <c r="G4" s="2" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="A5" s="25" t="inlineStr">
         <is>
           <t>TAG</t>
         </is>
       </c>
-      <c r="B5" s="10" t="n"/>
-      <c r="C5" s="15" t="inlineStr">
+      <c r="B5" s="22" t="n"/>
+      <c r="C5" s="25" t="inlineStr">
         <is>
           <t>Localização</t>
         </is>
       </c>
-      <c r="D5" s="9" t="n"/>
-      <c r="E5" s="10" t="n"/>
-      <c r="F5" s="15" t="inlineStr">
+      <c r="D5" s="21" t="n"/>
+      <c r="E5" s="22" t="n"/>
+      <c r="F5" s="25" t="inlineStr">
         <is>
           <t>Identificação</t>
         </is>
       </c>
-      <c r="G5" s="9" t="n"/>
-      <c r="H5" s="10" t="n"/>
-    </row>
-    <row r="6" ht="34.5" customHeight="1" s="14">
-      <c r="A6" s="30" t="inlineStr">
+      <c r="G5" s="21" t="n"/>
+      <c r="H5" s="22" t="n"/>
+    </row>
+    <row r="6" ht="34.5" customHeight="1" s="15">
+      <c r="A6" s="26" t="inlineStr">
         <is>
           <t>TT-SG-122104-01</t>
         </is>
       </c>
-      <c r="B6" s="10" t="n"/>
-      <c r="C6" s="30" t="inlineStr">
-        <is>
-          <t>PILAR</t>
-        </is>
-      </c>
-      <c r="D6" s="9" t="n"/>
-      <c r="E6" s="10" t="n"/>
-      <c r="F6" s="54" t="inlineStr">
-        <is>
-          <t>SAP: 123456</t>
-        </is>
-      </c>
-      <c r="G6" s="30" t="inlineStr">
-        <is>
-          <t>CE: 8902658</t>
-        </is>
-      </c>
-      <c r="H6" s="10" t="n"/>
-    </row>
-    <row r="7" ht="14.5" customHeight="1" s="14">
+      <c r="B6" s="22" t="n"/>
+      <c r="C6" s="26" t="inlineStr">
+        <is>
+          <t>teste</t>
+        </is>
+      </c>
+      <c r="D6" s="21" t="n"/>
+      <c r="E6" s="22" t="n"/>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>SAP: teste</t>
+        </is>
+      </c>
+      <c r="G6" s="26" t="inlineStr">
+        <is>
+          <t>CE: teste</t>
+        </is>
+      </c>
+      <c r="H6" s="22" t="n"/>
+    </row>
+    <row r="7" ht="14.5" customHeight="1" s="15">
       <c r="A7" s="2" t="n"/>
       <c r="B7" s="2" t="n"/>
       <c r="C7" s="2" t="n"/>
@@ -1042,97 +997,97 @@
       <c r="G7" s="3" t="n"/>
       <c r="H7" s="3" t="n"/>
     </row>
-    <row r="8" ht="14.5" customHeight="1" s="14">
-      <c r="A8" s="41" t="inlineStr">
+    <row r="8" ht="14.5" customHeight="1" s="15">
+      <c r="A8" s="27" t="inlineStr">
         <is>
           <t>OUTRAS INFORMAÇÕES (Descrição):</t>
         </is>
       </c>
-      <c r="B8" s="26" t="n"/>
-      <c r="C8" s="34" t="inlineStr">
+      <c r="B8" s="11" t="n"/>
+      <c r="C8" s="31" t="inlineStr">
         <is>
           <t>[ ] Transmissor de pressão estática (PT)</t>
         </is>
       </c>
-      <c r="D8" s="31" t="n"/>
-      <c r="E8" s="26" t="n"/>
-      <c r="F8" s="30" t="inlineStr">
-        <is>
-          <t>[ ] Termorresistência (TE)</t>
-        </is>
-      </c>
-      <c r="G8" s="31" t="n"/>
-      <c r="H8" s="26" t="n"/>
+      <c r="D8" s="13" t="n"/>
+      <c r="E8" s="11" t="n"/>
+      <c r="F8" s="26" t="inlineStr">
+        <is>
+          <t>[ ✔ ]Termorresistência (TE)</t>
+        </is>
+      </c>
+      <c r="G8" s="13" t="n"/>
+      <c r="H8" s="11" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="27" t="n"/>
-      <c r="B9" s="18" t="n"/>
-      <c r="C9" s="22" t="inlineStr">
+      <c r="A9" s="14" t="n"/>
+      <c r="B9" s="16" t="n"/>
+      <c r="C9" s="40" t="inlineStr">
         <is>
           <t>[ ] Transmissor de pressão diferencial (PDT)</t>
         </is>
       </c>
-      <c r="E9" s="18" t="n"/>
-      <c r="F9" s="27" t="n"/>
-      <c r="H9" s="18" t="n"/>
+      <c r="E9" s="16" t="n"/>
+      <c r="F9" s="14" t="n"/>
+      <c r="H9" s="16" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="28" t="n"/>
-      <c r="B10" s="29" t="n"/>
-      <c r="C10" s="44" t="inlineStr">
+      <c r="A10" s="17" t="n"/>
+      <c r="B10" s="19" t="n"/>
+      <c r="C10" s="23" t="inlineStr">
         <is>
           <t>[ ✔ ] Transmissor de temperatura (TT)</t>
         </is>
       </c>
-      <c r="D10" s="32" t="n"/>
-      <c r="E10" s="29" t="n"/>
-      <c r="F10" s="28" t="n"/>
-      <c r="G10" s="32" t="n"/>
-      <c r="H10" s="29" t="n"/>
+      <c r="D10" s="18" t="n"/>
+      <c r="E10" s="19" t="n"/>
+      <c r="F10" s="17" t="n"/>
+      <c r="G10" s="18" t="n"/>
+      <c r="H10" s="19" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="15" t="inlineStr">
+      <c r="A12" s="25" t="inlineStr">
         <is>
           <t>Nº do Certificado</t>
         </is>
       </c>
-      <c r="B12" s="9" t="n"/>
-      <c r="C12" s="10" t="n"/>
-      <c r="D12" s="35" t="inlineStr">
+      <c r="B12" s="21" t="n"/>
+      <c r="C12" s="22" t="n"/>
+      <c r="D12" s="32" t="inlineStr">
         <is>
           <t>Data da Calibração</t>
         </is>
       </c>
-      <c r="E12" s="36" t="n"/>
-      <c r="F12" s="12" t="n"/>
-      <c r="G12" s="11" t="inlineStr">
+      <c r="E12" s="33" t="n"/>
+      <c r="F12" s="34" t="n"/>
+      <c r="G12" s="41" t="inlineStr">
         <is>
           <t>Empresa Certificadora</t>
         </is>
       </c>
-      <c r="H12" s="12" t="n"/>
+      <c r="H12" s="34" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="30" t="inlineStr">
+      <c r="A13" s="26" t="inlineStr">
         <is>
           <t>25-ODS-0638 - TEM - 150</t>
         </is>
       </c>
-      <c r="B13" s="9" t="n"/>
-      <c r="C13" s="10" t="n"/>
-      <c r="D13" s="19" t="inlineStr">
+      <c r="B13" s="21" t="n"/>
+      <c r="C13" s="22" t="n"/>
+      <c r="D13" s="42" t="inlineStr">
         <is>
           <t>01/09/2025</t>
         </is>
       </c>
-      <c r="E13" s="20" t="n"/>
-      <c r="F13" s="21" t="n"/>
-      <c r="G13" s="38" t="inlineStr">
+      <c r="E13" s="43" t="n"/>
+      <c r="F13" s="37" t="n"/>
+      <c r="G13" s="36" t="inlineStr">
         <is>
           <t>ODS Lab</t>
         </is>
       </c>
-      <c r="H13" s="21" t="n"/>
+      <c r="H13" s="37" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n"/>
@@ -1145,527 +1100,527 @@
       <c r="H14" s="2" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="16" t="inlineStr">
+      <c r="A15" s="35" t="inlineStr">
         <is>
           <t>1 - ANÁLISE DO CERTIFICADO DE CALIBRAÇÃO</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="25" customHeight="1" s="14">
-      <c r="A16" s="33" t="inlineStr">
+    <row r="16" ht="25" customHeight="1" s="15">
+      <c r="A16" s="30" t="inlineStr">
         <is>
           <t>DESCRIÇÃO DOS ITENS A SEREM VERIFICADOS</t>
         </is>
       </c>
-      <c r="B16" s="9" t="n"/>
-      <c r="C16" s="9" t="n"/>
-      <c r="D16" s="9" t="n"/>
-      <c r="E16" s="10" t="n"/>
-      <c r="F16" s="33" t="inlineStr">
+      <c r="B16" s="21" t="n"/>
+      <c r="C16" s="21" t="n"/>
+      <c r="D16" s="21" t="n"/>
+      <c r="E16" s="22" t="n"/>
+      <c r="F16" s="30" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
       </c>
-      <c r="G16" s="33" t="inlineStr">
+      <c r="G16" s="30" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
-      <c r="H16" s="33" t="inlineStr">
+      <c r="H16" s="30" t="inlineStr">
         <is>
           <t>NÃO APLICÁVEL</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="16.5" customHeight="1" s="14">
-      <c r="A17" s="8" t="inlineStr">
+    <row r="17" ht="16.5" customHeight="1" s="15">
+      <c r="A17" s="20" t="inlineStr">
         <is>
           <t>a) Identificação unívoca (Número do Certificado de Calibração).</t>
         </is>
       </c>
-      <c r="B17" s="9" t="n"/>
-      <c r="C17" s="9" t="n"/>
-      <c r="D17" s="9" t="n"/>
-      <c r="E17" s="10" t="n"/>
-      <c r="F17" s="45" t="inlineStr">
-        <is>
-          <t>◉</t>
-        </is>
-      </c>
-      <c r="G17" s="45" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="H17" s="45" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="16.5" customHeight="1" s="14">
-      <c r="A18" s="8" t="inlineStr">
+      <c r="B17" s="21" t="n"/>
+      <c r="C17" s="21" t="n"/>
+      <c r="D17" s="21" t="n"/>
+      <c r="E17" s="22" t="n"/>
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>◉</t>
+        </is>
+      </c>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="16.5" customHeight="1" s="15">
+      <c r="A18" s="20" t="inlineStr">
         <is>
           <t>b) Nome e endereço do Laboratório/Empresa.</t>
         </is>
       </c>
-      <c r="B18" s="9" t="n"/>
-      <c r="C18" s="9" t="n"/>
-      <c r="D18" s="9" t="n"/>
-      <c r="E18" s="10" t="n"/>
-      <c r="F18" s="45" t="inlineStr">
-        <is>
-          <t>◉</t>
-        </is>
-      </c>
-      <c r="G18" s="45" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="H18" s="45" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="31" customHeight="1" s="14">
-      <c r="A19" s="8" t="inlineStr">
+      <c r="B18" s="21" t="n"/>
+      <c r="C18" s="21" t="n"/>
+      <c r="D18" s="21" t="n"/>
+      <c r="E18" s="22" t="n"/>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>◉</t>
+        </is>
+      </c>
+      <c r="G18" s="7" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="31" customHeight="1" s="15">
+      <c r="A19" s="20" t="inlineStr">
         <is>
           <t>c) Logotipo da RBC (para instrumento associado a sistemas de medição fiscal, apropriação, custódia, flare)</t>
         </is>
       </c>
-      <c r="B19" s="9" t="n"/>
-      <c r="C19" s="9" t="n"/>
-      <c r="D19" s="9" t="n"/>
-      <c r="E19" s="10" t="n"/>
-      <c r="F19" s="45" t="inlineStr">
-        <is>
-          <t>◉</t>
-        </is>
-      </c>
-      <c r="G19" s="45" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="H19" s="45" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="16.5" customHeight="1" s="14">
-      <c r="A20" s="8" t="inlineStr">
+      <c r="B19" s="21" t="n"/>
+      <c r="C19" s="21" t="n"/>
+      <c r="D19" s="21" t="n"/>
+      <c r="E19" s="22" t="n"/>
+      <c r="F19" s="7" t="inlineStr">
+        <is>
+          <t>◉</t>
+        </is>
+      </c>
+      <c r="G19" s="7" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="16.5" customHeight="1" s="15">
+      <c r="A20" s="20" t="inlineStr">
         <is>
           <t>d) Nome e endereço do cliente.</t>
         </is>
       </c>
-      <c r="B20" s="9" t="n"/>
-      <c r="C20" s="9" t="n"/>
-      <c r="D20" s="9" t="n"/>
-      <c r="E20" s="10" t="n"/>
-      <c r="F20" s="45" t="inlineStr">
-        <is>
-          <t>◉</t>
-        </is>
-      </c>
-      <c r="G20" s="45" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="H20" s="45" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="16.5" customHeight="1" s="14">
-      <c r="A21" s="8" t="inlineStr">
+      <c r="B20" s="21" t="n"/>
+      <c r="C20" s="21" t="n"/>
+      <c r="D20" s="21" t="n"/>
+      <c r="E20" s="22" t="n"/>
+      <c r="F20" s="7" t="inlineStr">
+        <is>
+          <t>◉</t>
+        </is>
+      </c>
+      <c r="G20" s="7" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="16.5" customHeight="1" s="15">
+      <c r="A21" s="20" t="inlineStr">
         <is>
           <t>e) Número de páginas e total de páginas.</t>
         </is>
       </c>
-      <c r="B21" s="9" t="n"/>
-      <c r="C21" s="9" t="n"/>
-      <c r="D21" s="9" t="n"/>
-      <c r="E21" s="10" t="n"/>
-      <c r="F21" s="45" t="inlineStr">
-        <is>
-          <t>◉</t>
-        </is>
-      </c>
-      <c r="G21" s="45" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="H21" s="45" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="16.5" customHeight="1" s="14">
-      <c r="A22" s="8" t="inlineStr">
+      <c r="B21" s="21" t="n"/>
+      <c r="C21" s="21" t="n"/>
+      <c r="D21" s="21" t="n"/>
+      <c r="E21" s="22" t="n"/>
+      <c r="F21" s="7" t="inlineStr">
+        <is>
+          <t>◉</t>
+        </is>
+      </c>
+      <c r="G21" s="7" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="16.5" customHeight="1" s="15">
+      <c r="A22" s="20" t="inlineStr">
         <is>
           <t>f) Identificação do método/procedimento utilizado.</t>
         </is>
       </c>
-      <c r="B22" s="9" t="n"/>
-      <c r="C22" s="9" t="n"/>
-      <c r="D22" s="9" t="n"/>
-      <c r="E22" s="10" t="n"/>
-      <c r="F22" s="45" t="inlineStr">
-        <is>
-          <t>◉</t>
-        </is>
-      </c>
-      <c r="G22" s="45" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="H22" s="45" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="16.5" customHeight="1" s="14">
-      <c r="A23" s="8" t="inlineStr">
+      <c r="B22" s="21" t="n"/>
+      <c r="C22" s="21" t="n"/>
+      <c r="D22" s="21" t="n"/>
+      <c r="E22" s="22" t="n"/>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>◉</t>
+        </is>
+      </c>
+      <c r="G22" s="7" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H22" s="7" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="16.5" customHeight="1" s="15">
+      <c r="A23" s="20" t="inlineStr">
         <is>
           <t>g) Registro das condições ambientais.</t>
         </is>
       </c>
-      <c r="B23" s="9" t="n"/>
-      <c r="C23" s="9" t="n"/>
-      <c r="D23" s="9" t="n"/>
-      <c r="E23" s="10" t="n"/>
-      <c r="F23" s="45" t="inlineStr">
-        <is>
-          <t>◉</t>
-        </is>
-      </c>
-      <c r="G23" s="45" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="H23" s="45" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="31" customHeight="1" s="14">
-      <c r="A24" s="8" t="inlineStr">
+      <c r="B23" s="21" t="n"/>
+      <c r="C23" s="21" t="n"/>
+      <c r="D23" s="21" t="n"/>
+      <c r="E23" s="22" t="n"/>
+      <c r="F23" s="7" t="inlineStr">
+        <is>
+          <t>◉</t>
+        </is>
+      </c>
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="31" customHeight="1" s="15">
+      <c r="A24" s="20" t="inlineStr">
         <is>
           <t>h) Descrição e identificação do item de calibração (ex.: nome, fabricante, tipo, modelo, número de série, outra identificação estabelecida pelo cliente).</t>
         </is>
       </c>
-      <c r="B24" s="9" t="n"/>
-      <c r="C24" s="9" t="n"/>
-      <c r="D24" s="9" t="n"/>
-      <c r="E24" s="10" t="n"/>
-      <c r="F24" s="45" t="inlineStr">
-        <is>
-          <t>◉</t>
-        </is>
-      </c>
-      <c r="G24" s="45" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="H24" s="45" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="16.5" customHeight="1" s="14">
-      <c r="A25" s="8" t="inlineStr">
+      <c r="B24" s="21" t="n"/>
+      <c r="C24" s="21" t="n"/>
+      <c r="D24" s="21" t="n"/>
+      <c r="E24" s="22" t="n"/>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>◉</t>
+        </is>
+      </c>
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H24" s="7" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="16.5" customHeight="1" s="15">
+      <c r="A25" s="20" t="inlineStr">
         <is>
           <t>i) A data do recebimento do(s) item(s) de calibração, se necessário.</t>
         </is>
       </c>
-      <c r="B25" s="9" t="n"/>
-      <c r="C25" s="9" t="n"/>
-      <c r="D25" s="9" t="n"/>
-      <c r="E25" s="10" t="n"/>
-      <c r="F25" s="45" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="G25" s="45" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="H25" s="45" t="inlineStr">
-        <is>
-          <t>◉</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="16.5" customHeight="1" s="14">
-      <c r="A26" s="8" t="inlineStr">
+      <c r="B25" s="21" t="n"/>
+      <c r="C25" s="21" t="n"/>
+      <c r="D25" s="21" t="n"/>
+      <c r="E25" s="22" t="n"/>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>◉</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="16.5" customHeight="1" s="15">
+      <c r="A26" s="20" t="inlineStr">
         <is>
           <t>j) A data da realização da calibração.</t>
         </is>
       </c>
-      <c r="B26" s="9" t="n"/>
-      <c r="C26" s="9" t="n"/>
-      <c r="D26" s="9" t="n"/>
-      <c r="E26" s="10" t="n"/>
-      <c r="F26" s="45" t="inlineStr">
-        <is>
-          <t>◉</t>
-        </is>
-      </c>
-      <c r="G26" s="45" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="H26" s="45" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="31" customHeight="1" s="14">
-      <c r="A27" s="8" t="inlineStr">
+      <c r="B26" s="21" t="n"/>
+      <c r="C26" s="21" t="n"/>
+      <c r="D26" s="21" t="n"/>
+      <c r="E26" s="22" t="n"/>
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>◉</t>
+        </is>
+      </c>
+      <c r="G26" s="7" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H26" s="7" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="31" customHeight="1" s="15">
+      <c r="A27" s="20" t="inlineStr">
         <is>
           <t>k) Os resultados da calibração estão com as unidades de medida no SI, onde apropriado.</t>
         </is>
       </c>
-      <c r="B27" s="9" t="n"/>
-      <c r="C27" s="9" t="n"/>
-      <c r="D27" s="9" t="n"/>
-      <c r="E27" s="10" t="n"/>
-      <c r="F27" s="45" t="inlineStr">
-        <is>
-          <t>◉</t>
-        </is>
-      </c>
-      <c r="G27" s="45" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="H27" s="45" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="16.5" customHeight="1" s="14">
-      <c r="A28" s="8" t="inlineStr">
+      <c r="B27" s="21" t="n"/>
+      <c r="C27" s="21" t="n"/>
+      <c r="D27" s="21" t="n"/>
+      <c r="E27" s="22" t="n"/>
+      <c r="F27" s="7" t="inlineStr">
+        <is>
+          <t>◉</t>
+        </is>
+      </c>
+      <c r="G27" s="7" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H27" s="7" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="16.5" customHeight="1" s="15">
+      <c r="A28" s="20" t="inlineStr">
         <is>
           <t>l) Evidências de que as medições são rastreáveis (Informações dos padrões utilizados).</t>
         </is>
       </c>
-      <c r="B28" s="9" t="n"/>
-      <c r="C28" s="9" t="n"/>
-      <c r="D28" s="9" t="n"/>
-      <c r="E28" s="10" t="n"/>
-      <c r="F28" s="45" t="inlineStr">
-        <is>
-          <t>◉</t>
-        </is>
-      </c>
-      <c r="G28" s="45" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="H28" s="45" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="31" customHeight="1" s="14">
-      <c r="A29" s="8" t="inlineStr">
+      <c r="B28" s="21" t="n"/>
+      <c r="C28" s="21" t="n"/>
+      <c r="D28" s="21" t="n"/>
+      <c r="E28" s="22" t="n"/>
+      <c r="F28" s="7" t="inlineStr">
+        <is>
+          <t>◉</t>
+        </is>
+      </c>
+      <c r="G28" s="7" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H28" s="7" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="31" customHeight="1" s="15">
+      <c r="A29" s="20" t="inlineStr">
         <is>
           <t>m) Nome(s), função (ões) e assinatura (s) ou identificações equivalentes das pessoas autorizadas para emissão do certificado.</t>
         </is>
       </c>
-      <c r="B29" s="9" t="n"/>
-      <c r="C29" s="9" t="n"/>
-      <c r="D29" s="9" t="n"/>
-      <c r="E29" s="10" t="n"/>
-      <c r="F29" s="45" t="inlineStr">
-        <is>
-          <t>◉</t>
-        </is>
-      </c>
-      <c r="G29" s="45" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="H29" s="45" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="31" customHeight="1" s="14">
-      <c r="A30" s="8" t="inlineStr">
+      <c r="B29" s="21" t="n"/>
+      <c r="C29" s="21" t="n"/>
+      <c r="D29" s="21" t="n"/>
+      <c r="E29" s="22" t="n"/>
+      <c r="F29" s="7" t="inlineStr">
+        <is>
+          <t>◉</t>
+        </is>
+      </c>
+      <c r="G29" s="7" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="31" customHeight="1" s="15">
+      <c r="A30" s="20" t="inlineStr">
         <is>
           <t>n) Declaração de que os resultados e incertezas se referem somente aos itens calibrados / inspecionados.</t>
         </is>
       </c>
-      <c r="B30" s="9" t="n"/>
-      <c r="C30" s="9" t="n"/>
-      <c r="D30" s="9" t="n"/>
-      <c r="E30" s="10" t="n"/>
-      <c r="F30" s="45" t="inlineStr">
-        <is>
-          <t>◉</t>
-        </is>
-      </c>
-      <c r="G30" s="45" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="H30" s="45" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="16.5" customHeight="1" s="14">
-      <c r="A31" s="8" t="inlineStr">
+      <c r="B30" s="21" t="n"/>
+      <c r="C30" s="21" t="n"/>
+      <c r="D30" s="21" t="n"/>
+      <c r="E30" s="22" t="n"/>
+      <c r="F30" s="7" t="inlineStr">
+        <is>
+          <t>◉</t>
+        </is>
+      </c>
+      <c r="G30" s="7" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H30" s="7" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="16.5" customHeight="1" s="15">
+      <c r="A31" s="20" t="inlineStr">
         <is>
           <t>o) Nível de confiança e fator de abrangência.</t>
         </is>
       </c>
-      <c r="B31" s="9" t="n"/>
-      <c r="C31" s="9" t="n"/>
-      <c r="D31" s="9" t="n"/>
-      <c r="E31" s="10" t="n"/>
-      <c r="F31" s="45" t="inlineStr">
-        <is>
-          <t>◉</t>
-        </is>
-      </c>
-      <c r="G31" s="45" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="H31" s="45" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="16.5" customHeight="1" s="14">
-      <c r="A32" s="8" t="inlineStr">
+      <c r="B31" s="21" t="n"/>
+      <c r="C31" s="21" t="n"/>
+      <c r="D31" s="21" t="n"/>
+      <c r="E31" s="22" t="n"/>
+      <c r="F31" s="7" t="inlineStr">
+        <is>
+          <t>◉</t>
+        </is>
+      </c>
+      <c r="G31" s="7" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H31" s="7" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="16.5" customHeight="1" s="15">
+      <c r="A32" s="20" t="inlineStr">
         <is>
           <t>p) Foi feita calibração de acordo com a faixa solicitada?</t>
         </is>
       </c>
-      <c r="B32" s="9" t="n"/>
-      <c r="C32" s="9" t="n"/>
-      <c r="D32" s="9" t="n"/>
-      <c r="E32" s="10" t="n"/>
-      <c r="F32" s="45" t="inlineStr">
-        <is>
-          <t>◉</t>
-        </is>
-      </c>
-      <c r="G32" s="45" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="H32" s="45" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="31" customHeight="1" s="14">
-      <c r="A33" s="8" t="inlineStr">
+      <c r="B32" s="21" t="n"/>
+      <c r="C32" s="21" t="n"/>
+      <c r="D32" s="21" t="n"/>
+      <c r="E32" s="22" t="n"/>
+      <c r="F32" s="7" t="inlineStr">
+        <is>
+          <t>◉</t>
+        </is>
+      </c>
+      <c r="G32" s="7" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H32" s="7" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="31" customHeight="1" s="15">
+      <c r="A33" s="20" t="inlineStr">
         <is>
           <t>q) Os erros máximos de medição (Erro sistemático remanescente + incerteza) são inferiores ao erro máximo admissível para o equipamento em questão?</t>
         </is>
       </c>
-      <c r="B33" s="9" t="n"/>
-      <c r="C33" s="9" t="n"/>
-      <c r="D33" s="9" t="n"/>
-      <c r="E33" s="10" t="n"/>
-      <c r="F33" s="45" t="inlineStr">
-        <is>
-          <t>◉</t>
-        </is>
-      </c>
-      <c r="G33" s="45" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="H33" s="45" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="31" customHeight="1" s="14">
-      <c r="A34" s="8" t="inlineStr">
+      <c r="B33" s="21" t="n"/>
+      <c r="C33" s="21" t="n"/>
+      <c r="D33" s="21" t="n"/>
+      <c r="E33" s="22" t="n"/>
+      <c r="F33" s="7" t="inlineStr">
+        <is>
+          <t>◉</t>
+        </is>
+      </c>
+      <c r="G33" s="7" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H33" s="7" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="31" customHeight="1" s="15">
+      <c r="A34" s="20" t="inlineStr">
         <is>
           <t>r) O instrumento está aprovado para o uso no ponto de medição a que se destina de acordo com os critérios de aceitação informados pelo cliente?</t>
         </is>
       </c>
-      <c r="B34" s="9" t="n"/>
-      <c r="C34" s="9" t="n"/>
-      <c r="D34" s="9" t="n"/>
-      <c r="E34" s="10" t="n"/>
-      <c r="F34" s="45" t="inlineStr">
-        <is>
-          <t>◉</t>
-        </is>
-      </c>
-      <c r="G34" s="45" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="H34" s="45" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="31" customHeight="1" s="14">
-      <c r="A35" s="8" t="inlineStr">
+      <c r="B34" s="21" t="n"/>
+      <c r="C34" s="21" t="n"/>
+      <c r="D34" s="21" t="n"/>
+      <c r="E34" s="22" t="n"/>
+      <c r="F34" s="7" t="inlineStr">
+        <is>
+          <t>◉</t>
+        </is>
+      </c>
+      <c r="G34" s="7" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H34" s="7" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="31" customHeight="1" s="15">
+      <c r="A35" s="20" t="inlineStr">
         <is>
           <t>s) No caso de ajuste no equipamento, estão informados os resultados das calibrações como encontrados (as found) e como deixados (as left)?</t>
         </is>
       </c>
-      <c r="B35" s="9" t="n"/>
-      <c r="C35" s="9" t="n"/>
-      <c r="D35" s="9" t="n"/>
-      <c r="E35" s="10" t="n"/>
-      <c r="F35" s="45" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="G35" s="45" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="H35" s="45" t="inlineStr">
+      <c r="B35" s="21" t="n"/>
+      <c r="C35" s="21" t="n"/>
+      <c r="D35" s="21" t="n"/>
+      <c r="E35" s="22" t="n"/>
+      <c r="F35" s="7" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="G35" s="7" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H35" s="7" t="inlineStr">
         <is>
           <t>◉</t>
         </is>
@@ -1678,83 +1633,80 @@
       <c r="H36" s="2" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="16" t="inlineStr">
+      <c r="A37" s="35" t="inlineStr">
         <is>
           <t>1.1 Conclusão da análise crítica do certificado de calibração:</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="23" t="inlineStr">
+      <c r="A38" s="28" t="inlineStr">
         <is>
           <t xml:space="preserve">O certificado está conforme e atende ao procedimento?  </t>
         </is>
       </c>
     </row>
-    <row r="39" ht="16.5" customHeight="1" s="14">
-      <c r="A39" s="13" t="inlineStr">
+    <row r="39" ht="16.5" customHeight="1" s="15">
+      <c r="A39" s="24" t="inlineStr">
         <is>
           <t>◉ Sim  ○ Não</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="13" t="n"/>
-      <c r="B40" s="13" t="n"/>
-      <c r="C40" s="13" t="n"/>
-      <c r="D40" s="13" t="n"/>
-      <c r="E40" s="13" t="n"/>
-      <c r="F40" s="13" t="n"/>
-      <c r="G40" s="13" t="n"/>
-      <c r="H40" s="13" t="n"/>
-      <c r="O40" s="7" t="n"/>
+      <c r="A40" s="24" t="n"/>
+      <c r="B40" s="24" t="n"/>
+      <c r="C40" s="24" t="n"/>
+      <c r="D40" s="24" t="n"/>
+      <c r="E40" s="24" t="n"/>
+      <c r="F40" s="24" t="n"/>
+      <c r="G40" s="24" t="n"/>
+      <c r="H40" s="24" t="n"/>
+      <c r="O40" s="6" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="16" t="inlineStr">
+      <c r="A41" s="35" t="inlineStr">
         <is>
           <t>OBSERVAÇÕES:</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="30" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <b val="1"/>
-            </rPr>
-            <t xml:space="preserve">Novo NS alterado no computador de vazão / XML / SFP
-</t>
-          </r>
-        </is>
-      </c>
-      <c r="B42" s="31" t="n"/>
-      <c r="C42" s="31" t="n"/>
-      <c r="D42" s="31" t="n"/>
-      <c r="E42" s="31" t="n"/>
-      <c r="F42" s="31" t="n"/>
-      <c r="G42" s="31" t="n"/>
-      <c r="H42" s="26" t="n"/>
+      <c r="A42" s="44" t="inlineStr"/>
+      <c r="B42" s="13" t="n"/>
+      <c r="C42" s="13" t="n"/>
+      <c r="D42" s="13" t="n"/>
+      <c r="E42" s="13" t="n"/>
+      <c r="F42" s="13" t="n"/>
+      <c r="G42" s="13" t="n"/>
+      <c r="H42" s="11" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="28" t="n"/>
-      <c r="B43" s="32" t="n"/>
-      <c r="C43" s="32" t="n"/>
-      <c r="D43" s="32" t="n"/>
-      <c r="E43" s="32" t="n"/>
-      <c r="F43" s="32" t="n"/>
-      <c r="G43" s="32" t="n"/>
-      <c r="H43" s="29" t="n"/>
+      <c r="A43" s="17" t="n"/>
+      <c r="B43" s="18" t="n"/>
+      <c r="C43" s="18" t="n"/>
+      <c r="D43" s="18" t="n"/>
+      <c r="E43" s="18" t="n"/>
+      <c r="F43" s="18" t="n"/>
+      <c r="G43" s="18" t="n"/>
+      <c r="H43" s="19" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="61" t="inlineStr">
+      <c r="A45" s="45" t="n"/>
+      <c r="B45" s="45" t="n"/>
+      <c r="C45" s="45" t="n"/>
+      <c r="D45" s="46" t="inlineStr">
         <is>
           <t>Data: 12/09/2025</t>
         </is>
       </c>
+      <c r="E45" s="45" t="n"/>
+      <c r="F45" s="45" t="n"/>
+      <c r="G45" s="45" t="n"/>
+      <c r="H45" s="45" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="13" t="inlineStr">
+      <c r="A46" s="24" t="inlineStr">
         <is>
           <t>_____________________________________</t>
         </is>
@@ -1763,14 +1715,14 @@
     <row r="47"/>
     <row r="48"/>
     <row r="49">
-      <c r="A49" s="23" t="inlineStr">
+      <c r="A49" s="28" t="inlineStr">
         <is>
           <t>Responsável pela Análise</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="51">
+  <mergeCells count="50">
     <mergeCell ref="A30:E30"/>
     <mergeCell ref="A34:E34"/>
     <mergeCell ref="G12:H12"/>
@@ -1782,7 +1734,6 @@
     <mergeCell ref="A15:H15"/>
     <mergeCell ref="C9:E9"/>
     <mergeCell ref="A49:H49"/>
-    <mergeCell ref="A45:H45"/>
     <mergeCell ref="A12:C12"/>
     <mergeCell ref="A1:B3"/>
     <mergeCell ref="A6:B6"/>
@@ -1797,8 +1748,8 @@
     <mergeCell ref="G13:H13"/>
     <mergeCell ref="A37:H37"/>
     <mergeCell ref="G3:H3"/>
+    <mergeCell ref="A27:E27"/>
     <mergeCell ref="A18:E18"/>
-    <mergeCell ref="A27:E27"/>
     <mergeCell ref="A21:E21"/>
     <mergeCell ref="A13:C13"/>
     <mergeCell ref="A26:E26"/>

</xml_diff>

<commit_message>
ajuste template AC origem + correção TE+TT
</commit_message>
<xml_diff>
--- a/TemplateAC_ORIGEM.xlsx
+++ b/TemplateAC_ORIGEM.xlsx
@@ -399,77 +399,77 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -885,109 +885,109 @@
   <dimension ref="A1:O49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
-    <col width="15" customWidth="1" style="15" min="1" max="4"/>
-    <col width="11.7265625" customWidth="1" style="15" min="5" max="5"/>
-    <col width="12.453125" customWidth="1" style="15" min="6" max="6"/>
-    <col width="10" customWidth="1" style="15" min="7" max="7"/>
-    <col width="15" customWidth="1" style="15" min="8" max="8"/>
+    <col width="15" customWidth="1" style="19" min="1" max="4"/>
+    <col width="11.7265625" customWidth="1" style="19" min="5" max="5"/>
+    <col width="12.453125" customWidth="1" style="19" min="6" max="6"/>
+    <col width="4.90625" bestFit="1" customWidth="1" style="19" min="7" max="7"/>
+    <col width="15" customWidth="1" style="19" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20" customHeight="1" s="15">
-      <c r="A1" s="29" t="n"/>
-      <c r="B1" s="11" t="n"/>
-      <c r="C1" s="12" t="inlineStr">
+    <row r="1" ht="20" customHeight="1" s="19">
+      <c r="A1" s="26" t="n"/>
+      <c r="B1" s="27" t="n"/>
+      <c r="C1" s="43" t="inlineStr">
         <is>
           <t>REGISTRO DE ANÁLISE CRÍTICA DE CERTIFICADO DE CALIBRAÇÃO DE SECUNDÁRIOS</t>
         </is>
       </c>
-      <c r="D1" s="13" t="n"/>
-      <c r="E1" s="13" t="n"/>
-      <c r="F1" s="11" t="n"/>
-      <c r="G1" s="10" t="inlineStr">
+      <c r="D1" s="33" t="n"/>
+      <c r="E1" s="33" t="n"/>
+      <c r="F1" s="27" t="n"/>
+      <c r="G1" s="42" t="inlineStr">
         <is>
           <t>FO-COR-GER-CPROD-030</t>
         </is>
       </c>
-      <c r="H1" s="11" t="n"/>
-    </row>
-    <row r="2" ht="20" customHeight="1" s="15">
-      <c r="A2" s="14" t="n"/>
-      <c r="B2" s="16" t="n"/>
-      <c r="C2" s="14" t="n"/>
-      <c r="F2" s="16" t="n"/>
-      <c r="G2" s="39" t="inlineStr">
+      <c r="H1" s="27" t="n"/>
+    </row>
+    <row r="2" ht="20" customHeight="1" s="19">
+      <c r="A2" s="28" t="n"/>
+      <c r="B2" s="22" t="n"/>
+      <c r="C2" s="28" t="n"/>
+      <c r="F2" s="22" t="n"/>
+      <c r="G2" s="21" t="inlineStr">
         <is>
           <t>Revisão: 0</t>
         </is>
       </c>
-      <c r="H2" s="16" t="n"/>
-    </row>
-    <row r="3" ht="20" customHeight="1" s="15">
-      <c r="A3" s="17" t="n"/>
-      <c r="B3" s="19" t="n"/>
-      <c r="C3" s="17" t="n"/>
-      <c r="D3" s="18" t="n"/>
-      <c r="E3" s="18" t="n"/>
-      <c r="F3" s="19" t="n"/>
-      <c r="G3" s="38" t="inlineStr">
+      <c r="H2" s="22" t="n"/>
+    </row>
+    <row r="3" ht="20" customHeight="1" s="19">
+      <c r="A3" s="29" t="n"/>
+      <c r="B3" s="30" t="n"/>
+      <c r="C3" s="29" t="n"/>
+      <c r="D3" s="34" t="n"/>
+      <c r="E3" s="34" t="n"/>
+      <c r="F3" s="30" t="n"/>
+      <c r="G3" s="40" t="inlineStr">
         <is>
           <t>Página: 1/1</t>
         </is>
       </c>
-      <c r="H3" s="19" t="n"/>
+      <c r="H3" s="30" t="n"/>
     </row>
     <row r="4">
       <c r="G4" s="2" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="25" t="inlineStr">
+      <c r="A5" s="20" t="inlineStr">
         <is>
           <t>TAG</t>
         </is>
       </c>
-      <c r="B5" s="22" t="n"/>
-      <c r="C5" s="25" t="inlineStr">
+      <c r="B5" s="12" t="n"/>
+      <c r="C5" s="20" t="inlineStr">
         <is>
           <t>Localização</t>
         </is>
       </c>
-      <c r="D5" s="21" t="n"/>
-      <c r="E5" s="22" t="n"/>
-      <c r="F5" s="25" t="inlineStr">
+      <c r="D5" s="11" t="n"/>
+      <c r="E5" s="12" t="n"/>
+      <c r="F5" s="20" t="inlineStr">
         <is>
           <t>Identificação</t>
         </is>
       </c>
-      <c r="G5" s="21" t="n"/>
-      <c r="H5" s="22" t="n"/>
-    </row>
-    <row r="6" ht="34.5" customHeight="1" s="15">
-      <c r="A6" s="26" t="inlineStr">
+      <c r="G5" s="11" t="n"/>
+      <c r="H5" s="12" t="n"/>
+    </row>
+    <row r="6" ht="34.5" customHeight="1" s="19">
+      <c r="A6" s="31" t="inlineStr">
         <is>
           <t>TT-SG-122104-01</t>
         </is>
       </c>
-      <c r="B6" s="22" t="n"/>
-      <c r="C6" s="26" t="inlineStr">
+      <c r="B6" s="12" t="n"/>
+      <c r="C6" s="31" t="inlineStr">
         <is>
           <t>teste</t>
         </is>
       </c>
-      <c r="D6" s="21" t="n"/>
-      <c r="E6" s="22" t="n"/>
+      <c r="D6" s="11" t="n"/>
+      <c r="E6" s="12" t="n"/>
       <c r="F6" s="8" t="inlineStr">
         <is>
           <t>SAP: teste</t>
         </is>
       </c>
-      <c r="G6" s="26" t="inlineStr">
+      <c r="G6" s="31" t="inlineStr">
         <is>
           <t>CE: teste</t>
         </is>
       </c>
-      <c r="H6" s="22" t="n"/>
-    </row>
-    <row r="7" ht="14.5" customHeight="1" s="15">
+      <c r="H6" s="12" t="n"/>
+    </row>
+    <row r="7" ht="14.5" customHeight="1" s="19">
       <c r="A7" s="2" t="n"/>
       <c r="B7" s="2" t="n"/>
       <c r="C7" s="2" t="n"/>
@@ -997,97 +997,97 @@
       <c r="G7" s="3" t="n"/>
       <c r="H7" s="3" t="n"/>
     </row>
-    <row r="8" ht="14.5" customHeight="1" s="15">
-      <c r="A8" s="27" t="inlineStr">
+    <row r="8" ht="14.5" customHeight="1" s="19">
+      <c r="A8" s="41" t="inlineStr">
         <is>
           <t>OUTRAS INFORMAÇÕES (Descrição):</t>
         </is>
       </c>
-      <c r="B8" s="11" t="n"/>
-      <c r="C8" s="31" t="inlineStr">
+      <c r="B8" s="27" t="n"/>
+      <c r="C8" s="36" t="inlineStr">
         <is>
           <t>[ ] Transmissor de pressão estática (PT)</t>
         </is>
       </c>
-      <c r="D8" s="13" t="n"/>
-      <c r="E8" s="11" t="n"/>
-      <c r="F8" s="26" t="inlineStr">
+      <c r="D8" s="33" t="n"/>
+      <c r="E8" s="27" t="n"/>
+      <c r="F8" s="31" t="inlineStr">
         <is>
           <t>[ ✔ ]Termorresistência (TE)</t>
         </is>
       </c>
-      <c r="G8" s="13" t="n"/>
-      <c r="H8" s="11" t="n"/>
+      <c r="G8" s="33" t="n"/>
+      <c r="H8" s="27" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="14" t="n"/>
-      <c r="B9" s="16" t="n"/>
-      <c r="C9" s="40" t="inlineStr">
+      <c r="A9" s="28" t="n"/>
+      <c r="B9" s="22" t="n"/>
+      <c r="C9" s="24" t="inlineStr">
         <is>
           <t>[ ] Transmissor de pressão diferencial (PDT)</t>
         </is>
       </c>
-      <c r="E9" s="16" t="n"/>
-      <c r="F9" s="14" t="n"/>
-      <c r="H9" s="16" t="n"/>
+      <c r="E9" s="22" t="n"/>
+      <c r="F9" s="28" t="n"/>
+      <c r="H9" s="22" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="17" t="n"/>
-      <c r="B10" s="19" t="n"/>
-      <c r="C10" s="23" t="inlineStr">
+      <c r="A10" s="29" t="n"/>
+      <c r="B10" s="30" t="n"/>
+      <c r="C10" s="44" t="inlineStr">
         <is>
           <t>[ ✔ ] Transmissor de temperatura (TT)</t>
         </is>
       </c>
-      <c r="D10" s="18" t="n"/>
-      <c r="E10" s="19" t="n"/>
-      <c r="F10" s="17" t="n"/>
-      <c r="G10" s="18" t="n"/>
-      <c r="H10" s="19" t="n"/>
+      <c r="D10" s="34" t="n"/>
+      <c r="E10" s="30" t="n"/>
+      <c r="F10" s="29" t="n"/>
+      <c r="G10" s="34" t="n"/>
+      <c r="H10" s="30" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="25" t="inlineStr">
+      <c r="A12" s="20" t="inlineStr">
         <is>
           <t>Nº do Certificado</t>
         </is>
       </c>
-      <c r="B12" s="21" t="n"/>
-      <c r="C12" s="22" t="n"/>
-      <c r="D12" s="32" t="inlineStr">
+      <c r="B12" s="11" t="n"/>
+      <c r="C12" s="12" t="n"/>
+      <c r="D12" s="37" t="inlineStr">
         <is>
           <t>Data da Calibração</t>
         </is>
       </c>
-      <c r="E12" s="33" t="n"/>
-      <c r="F12" s="34" t="n"/>
-      <c r="G12" s="41" t="inlineStr">
+      <c r="E12" s="38" t="n"/>
+      <c r="F12" s="14" t="n"/>
+      <c r="G12" s="13" t="inlineStr">
         <is>
           <t>Empresa Certificadora</t>
         </is>
       </c>
-      <c r="H12" s="34" t="n"/>
+      <c r="H12" s="14" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="26" t="inlineStr">
+      <c r="A13" s="31" t="inlineStr">
         <is>
           <t>25-ODS-0638 - TEM - 150</t>
         </is>
       </c>
-      <c r="B13" s="21" t="n"/>
-      <c r="C13" s="22" t="n"/>
-      <c r="D13" s="42" t="inlineStr">
+      <c r="B13" s="11" t="n"/>
+      <c r="C13" s="12" t="n"/>
+      <c r="D13" s="15" t="inlineStr">
         <is>
           <t>01/09/2025</t>
         </is>
       </c>
-      <c r="E13" s="43" t="n"/>
-      <c r="F13" s="37" t="n"/>
-      <c r="G13" s="36" t="inlineStr">
+      <c r="E13" s="16" t="n"/>
+      <c r="F13" s="17" t="n"/>
+      <c r="G13" s="39" t="inlineStr">
         <is>
           <t>ODS Lab</t>
         </is>
       </c>
-      <c r="H13" s="37" t="n"/>
+      <c r="H13" s="17" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n"/>
@@ -1100,48 +1100,48 @@
       <c r="H14" s="2" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="35" t="inlineStr">
+      <c r="A15" s="23" t="inlineStr">
         <is>
           <t>1 - ANÁLISE DO CERTIFICADO DE CALIBRAÇÃO</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="25" customHeight="1" s="15">
-      <c r="A16" s="30" t="inlineStr">
+    <row r="16" ht="25" customHeight="1" s="19">
+      <c r="A16" s="35" t="inlineStr">
         <is>
           <t>DESCRIÇÃO DOS ITENS A SEREM VERIFICADOS</t>
         </is>
       </c>
-      <c r="B16" s="21" t="n"/>
-      <c r="C16" s="21" t="n"/>
-      <c r="D16" s="21" t="n"/>
-      <c r="E16" s="22" t="n"/>
-      <c r="F16" s="30" t="inlineStr">
+      <c r="B16" s="11" t="n"/>
+      <c r="C16" s="11" t="n"/>
+      <c r="D16" s="11" t="n"/>
+      <c r="E16" s="12" t="n"/>
+      <c r="F16" s="35" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
       </c>
-      <c r="G16" s="30" t="inlineStr">
+      <c r="G16" s="35" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
-      <c r="H16" s="30" t="inlineStr">
+      <c r="H16" s="35" t="inlineStr">
         <is>
           <t>NÃO APLICÁVEL</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="16.5" customHeight="1" s="15">
-      <c r="A17" s="20" t="inlineStr">
+    <row r="17" ht="16.5" customHeight="1" s="19">
+      <c r="A17" s="10" t="inlineStr">
         <is>
           <t>a) Identificação unívoca (Número do Certificado de Calibração).</t>
         </is>
       </c>
-      <c r="B17" s="21" t="n"/>
-      <c r="C17" s="21" t="n"/>
-      <c r="D17" s="21" t="n"/>
-      <c r="E17" s="22" t="n"/>
+      <c r="B17" s="11" t="n"/>
+      <c r="C17" s="11" t="n"/>
+      <c r="D17" s="11" t="n"/>
+      <c r="E17" s="12" t="n"/>
       <c r="F17" s="7" t="inlineStr">
         <is>
           <t>◉</t>
@@ -1158,16 +1158,16 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="16.5" customHeight="1" s="15">
-      <c r="A18" s="20" t="inlineStr">
+    <row r="18" ht="16.5" customHeight="1" s="19">
+      <c r="A18" s="10" t="inlineStr">
         <is>
           <t>b) Nome e endereço do Laboratório/Empresa.</t>
         </is>
       </c>
-      <c r="B18" s="21" t="n"/>
-      <c r="C18" s="21" t="n"/>
-      <c r="D18" s="21" t="n"/>
-      <c r="E18" s="22" t="n"/>
+      <c r="B18" s="11" t="n"/>
+      <c r="C18" s="11" t="n"/>
+      <c r="D18" s="11" t="n"/>
+      <c r="E18" s="12" t="n"/>
       <c r="F18" s="7" t="inlineStr">
         <is>
           <t>◉</t>
@@ -1184,16 +1184,16 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="31" customHeight="1" s="15">
-      <c r="A19" s="20" t="inlineStr">
+    <row r="19" ht="31" customHeight="1" s="19">
+      <c r="A19" s="10" t="inlineStr">
         <is>
           <t>c) Logotipo da RBC (para instrumento associado a sistemas de medição fiscal, apropriação, custódia, flare)</t>
         </is>
       </c>
-      <c r="B19" s="21" t="n"/>
-      <c r="C19" s="21" t="n"/>
-      <c r="D19" s="21" t="n"/>
-      <c r="E19" s="22" t="n"/>
+      <c r="B19" s="11" t="n"/>
+      <c r="C19" s="11" t="n"/>
+      <c r="D19" s="11" t="n"/>
+      <c r="E19" s="12" t="n"/>
       <c r="F19" s="7" t="inlineStr">
         <is>
           <t>◉</t>
@@ -1210,16 +1210,16 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="16.5" customHeight="1" s="15">
-      <c r="A20" s="20" t="inlineStr">
+    <row r="20" ht="16.5" customHeight="1" s="19">
+      <c r="A20" s="10" t="inlineStr">
         <is>
           <t>d) Nome e endereço do cliente.</t>
         </is>
       </c>
-      <c r="B20" s="21" t="n"/>
-      <c r="C20" s="21" t="n"/>
-      <c r="D20" s="21" t="n"/>
-      <c r="E20" s="22" t="n"/>
+      <c r="B20" s="11" t="n"/>
+      <c r="C20" s="11" t="n"/>
+      <c r="D20" s="11" t="n"/>
+      <c r="E20" s="12" t="n"/>
       <c r="F20" s="7" t="inlineStr">
         <is>
           <t>◉</t>
@@ -1236,16 +1236,16 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="16.5" customHeight="1" s="15">
-      <c r="A21" s="20" t="inlineStr">
+    <row r="21" ht="16.5" customHeight="1" s="19">
+      <c r="A21" s="10" t="inlineStr">
         <is>
           <t>e) Número de páginas e total de páginas.</t>
         </is>
       </c>
-      <c r="B21" s="21" t="n"/>
-      <c r="C21" s="21" t="n"/>
-      <c r="D21" s="21" t="n"/>
-      <c r="E21" s="22" t="n"/>
+      <c r="B21" s="11" t="n"/>
+      <c r="C21" s="11" t="n"/>
+      <c r="D21" s="11" t="n"/>
+      <c r="E21" s="12" t="n"/>
       <c r="F21" s="7" t="inlineStr">
         <is>
           <t>◉</t>
@@ -1262,16 +1262,16 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="16.5" customHeight="1" s="15">
-      <c r="A22" s="20" t="inlineStr">
+    <row r="22" ht="16.5" customHeight="1" s="19">
+      <c r="A22" s="10" t="inlineStr">
         <is>
           <t>f) Identificação do método/procedimento utilizado.</t>
         </is>
       </c>
-      <c r="B22" s="21" t="n"/>
-      <c r="C22" s="21" t="n"/>
-      <c r="D22" s="21" t="n"/>
-      <c r="E22" s="22" t="n"/>
+      <c r="B22" s="11" t="n"/>
+      <c r="C22" s="11" t="n"/>
+      <c r="D22" s="11" t="n"/>
+      <c r="E22" s="12" t="n"/>
       <c r="F22" s="7" t="inlineStr">
         <is>
           <t>◉</t>
@@ -1288,16 +1288,16 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="16.5" customHeight="1" s="15">
-      <c r="A23" s="20" t="inlineStr">
+    <row r="23" ht="16.5" customHeight="1" s="19">
+      <c r="A23" s="10" t="inlineStr">
         <is>
           <t>g) Registro das condições ambientais.</t>
         </is>
       </c>
-      <c r="B23" s="21" t="n"/>
-      <c r="C23" s="21" t="n"/>
-      <c r="D23" s="21" t="n"/>
-      <c r="E23" s="22" t="n"/>
+      <c r="B23" s="11" t="n"/>
+      <c r="C23" s="11" t="n"/>
+      <c r="D23" s="11" t="n"/>
+      <c r="E23" s="12" t="n"/>
       <c r="F23" s="7" t="inlineStr">
         <is>
           <t>◉</t>
@@ -1314,16 +1314,16 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="31" customHeight="1" s="15">
-      <c r="A24" s="20" t="inlineStr">
+    <row r="24" ht="31" customHeight="1" s="19">
+      <c r="A24" s="10" t="inlineStr">
         <is>
           <t>h) Descrição e identificação do item de calibração (ex.: nome, fabricante, tipo, modelo, número de série, outra identificação estabelecida pelo cliente).</t>
         </is>
       </c>
-      <c r="B24" s="21" t="n"/>
-      <c r="C24" s="21" t="n"/>
-      <c r="D24" s="21" t="n"/>
-      <c r="E24" s="22" t="n"/>
+      <c r="B24" s="11" t="n"/>
+      <c r="C24" s="11" t="n"/>
+      <c r="D24" s="11" t="n"/>
+      <c r="E24" s="12" t="n"/>
       <c r="F24" s="7" t="inlineStr">
         <is>
           <t>◉</t>
@@ -1340,16 +1340,16 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="16.5" customHeight="1" s="15">
-      <c r="A25" s="20" t="inlineStr">
+    <row r="25" ht="16.5" customHeight="1" s="19">
+      <c r="A25" s="10" t="inlineStr">
         <is>
           <t>i) A data do recebimento do(s) item(s) de calibração, se necessário.</t>
         </is>
       </c>
-      <c r="B25" s="21" t="n"/>
-      <c r="C25" s="21" t="n"/>
-      <c r="D25" s="21" t="n"/>
-      <c r="E25" s="22" t="n"/>
+      <c r="B25" s="11" t="n"/>
+      <c r="C25" s="11" t="n"/>
+      <c r="D25" s="11" t="n"/>
+      <c r="E25" s="12" t="n"/>
       <c r="F25" s="7" t="inlineStr">
         <is>
           <t>○</t>
@@ -1366,16 +1366,16 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="16.5" customHeight="1" s="15">
-      <c r="A26" s="20" t="inlineStr">
+    <row r="26" ht="16.5" customHeight="1" s="19">
+      <c r="A26" s="10" t="inlineStr">
         <is>
           <t>j) A data da realização da calibração.</t>
         </is>
       </c>
-      <c r="B26" s="21" t="n"/>
-      <c r="C26" s="21" t="n"/>
-      <c r="D26" s="21" t="n"/>
-      <c r="E26" s="22" t="n"/>
+      <c r="B26" s="11" t="n"/>
+      <c r="C26" s="11" t="n"/>
+      <c r="D26" s="11" t="n"/>
+      <c r="E26" s="12" t="n"/>
       <c r="F26" s="7" t="inlineStr">
         <is>
           <t>◉</t>
@@ -1392,16 +1392,16 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="31" customHeight="1" s="15">
-      <c r="A27" s="20" t="inlineStr">
+    <row r="27" ht="31" customHeight="1" s="19">
+      <c r="A27" s="10" t="inlineStr">
         <is>
           <t>k) Os resultados da calibração estão com as unidades de medida no SI, onde apropriado.</t>
         </is>
       </c>
-      <c r="B27" s="21" t="n"/>
-      <c r="C27" s="21" t="n"/>
-      <c r="D27" s="21" t="n"/>
-      <c r="E27" s="22" t="n"/>
+      <c r="B27" s="11" t="n"/>
+      <c r="C27" s="11" t="n"/>
+      <c r="D27" s="11" t="n"/>
+      <c r="E27" s="12" t="n"/>
       <c r="F27" s="7" t="inlineStr">
         <is>
           <t>◉</t>
@@ -1418,16 +1418,16 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="16.5" customHeight="1" s="15">
-      <c r="A28" s="20" t="inlineStr">
+    <row r="28" ht="16.5" customHeight="1" s="19">
+      <c r="A28" s="10" t="inlineStr">
         <is>
           <t>l) Evidências de que as medições são rastreáveis (Informações dos padrões utilizados).</t>
         </is>
       </c>
-      <c r="B28" s="21" t="n"/>
-      <c r="C28" s="21" t="n"/>
-      <c r="D28" s="21" t="n"/>
-      <c r="E28" s="22" t="n"/>
+      <c r="B28" s="11" t="n"/>
+      <c r="C28" s="11" t="n"/>
+      <c r="D28" s="11" t="n"/>
+      <c r="E28" s="12" t="n"/>
       <c r="F28" s="7" t="inlineStr">
         <is>
           <t>◉</t>
@@ -1444,16 +1444,16 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="31" customHeight="1" s="15">
-      <c r="A29" s="20" t="inlineStr">
+    <row r="29" ht="31" customHeight="1" s="19">
+      <c r="A29" s="10" t="inlineStr">
         <is>
           <t>m) Nome(s), função (ões) e assinatura (s) ou identificações equivalentes das pessoas autorizadas para emissão do certificado.</t>
         </is>
       </c>
-      <c r="B29" s="21" t="n"/>
-      <c r="C29" s="21" t="n"/>
-      <c r="D29" s="21" t="n"/>
-      <c r="E29" s="22" t="n"/>
+      <c r="B29" s="11" t="n"/>
+      <c r="C29" s="11" t="n"/>
+      <c r="D29" s="11" t="n"/>
+      <c r="E29" s="12" t="n"/>
       <c r="F29" s="7" t="inlineStr">
         <is>
           <t>◉</t>
@@ -1470,16 +1470,16 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="31" customHeight="1" s="15">
-      <c r="A30" s="20" t="inlineStr">
+    <row r="30" ht="31" customHeight="1" s="19">
+      <c r="A30" s="10" t="inlineStr">
         <is>
           <t>n) Declaração de que os resultados e incertezas se referem somente aos itens calibrados / inspecionados.</t>
         </is>
       </c>
-      <c r="B30" s="21" t="n"/>
-      <c r="C30" s="21" t="n"/>
-      <c r="D30" s="21" t="n"/>
-      <c r="E30" s="22" t="n"/>
+      <c r="B30" s="11" t="n"/>
+      <c r="C30" s="11" t="n"/>
+      <c r="D30" s="11" t="n"/>
+      <c r="E30" s="12" t="n"/>
       <c r="F30" s="7" t="inlineStr">
         <is>
           <t>◉</t>
@@ -1496,16 +1496,16 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="16.5" customHeight="1" s="15">
-      <c r="A31" s="20" t="inlineStr">
+    <row r="31" ht="16.5" customHeight="1" s="19">
+      <c r="A31" s="10" t="inlineStr">
         <is>
           <t>o) Nível de confiança e fator de abrangência.</t>
         </is>
       </c>
-      <c r="B31" s="21" t="n"/>
-      <c r="C31" s="21" t="n"/>
-      <c r="D31" s="21" t="n"/>
-      <c r="E31" s="22" t="n"/>
+      <c r="B31" s="11" t="n"/>
+      <c r="C31" s="11" t="n"/>
+      <c r="D31" s="11" t="n"/>
+      <c r="E31" s="12" t="n"/>
       <c r="F31" s="7" t="inlineStr">
         <is>
           <t>◉</t>
@@ -1522,16 +1522,16 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="16.5" customHeight="1" s="15">
-      <c r="A32" s="20" t="inlineStr">
+    <row r="32" ht="16.5" customHeight="1" s="19">
+      <c r="A32" s="10" t="inlineStr">
         <is>
           <t>p) Foi feita calibração de acordo com a faixa solicitada?</t>
         </is>
       </c>
-      <c r="B32" s="21" t="n"/>
-      <c r="C32" s="21" t="n"/>
-      <c r="D32" s="21" t="n"/>
-      <c r="E32" s="22" t="n"/>
+      <c r="B32" s="11" t="n"/>
+      <c r="C32" s="11" t="n"/>
+      <c r="D32" s="11" t="n"/>
+      <c r="E32" s="12" t="n"/>
       <c r="F32" s="7" t="inlineStr">
         <is>
           <t>◉</t>
@@ -1548,16 +1548,16 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="31" customHeight="1" s="15">
-      <c r="A33" s="20" t="inlineStr">
+    <row r="33" ht="31" customHeight="1" s="19">
+      <c r="A33" s="10" t="inlineStr">
         <is>
           <t>q) Os erros máximos de medição (Erro sistemático remanescente + incerteza) são inferiores ao erro máximo admissível para o equipamento em questão?</t>
         </is>
       </c>
-      <c r="B33" s="21" t="n"/>
-      <c r="C33" s="21" t="n"/>
-      <c r="D33" s="21" t="n"/>
-      <c r="E33" s="22" t="n"/>
+      <c r="B33" s="11" t="n"/>
+      <c r="C33" s="11" t="n"/>
+      <c r="D33" s="11" t="n"/>
+      <c r="E33" s="12" t="n"/>
       <c r="F33" s="7" t="inlineStr">
         <is>
           <t>◉</t>
@@ -1574,16 +1574,16 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="31" customHeight="1" s="15">
-      <c r="A34" s="20" t="inlineStr">
+    <row r="34" ht="31" customHeight="1" s="19">
+      <c r="A34" s="10" t="inlineStr">
         <is>
           <t>r) O instrumento está aprovado para o uso no ponto de medição a que se destina de acordo com os critérios de aceitação informados pelo cliente?</t>
         </is>
       </c>
-      <c r="B34" s="21" t="n"/>
-      <c r="C34" s="21" t="n"/>
-      <c r="D34" s="21" t="n"/>
-      <c r="E34" s="22" t="n"/>
+      <c r="B34" s="11" t="n"/>
+      <c r="C34" s="11" t="n"/>
+      <c r="D34" s="11" t="n"/>
+      <c r="E34" s="12" t="n"/>
       <c r="F34" s="7" t="inlineStr">
         <is>
           <t>◉</t>
@@ -1600,16 +1600,16 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="31" customHeight="1" s="15">
-      <c r="A35" s="20" t="inlineStr">
+    <row r="35" ht="31" customHeight="1" s="19">
+      <c r="A35" s="10" t="inlineStr">
         <is>
           <t>s) No caso de ajuste no equipamento, estão informados os resultados das calibrações como encontrados (as found) e como deixados (as left)?</t>
         </is>
       </c>
-      <c r="B35" s="21" t="n"/>
-      <c r="C35" s="21" t="n"/>
-      <c r="D35" s="21" t="n"/>
-      <c r="E35" s="22" t="n"/>
+      <c r="B35" s="11" t="n"/>
+      <c r="C35" s="11" t="n"/>
+      <c r="D35" s="11" t="n"/>
+      <c r="E35" s="12" t="n"/>
       <c r="F35" s="7" t="inlineStr">
         <is>
           <t>○</t>
@@ -1633,63 +1633,63 @@
       <c r="H36" s="2" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="35" t="inlineStr">
+      <c r="A37" s="23" t="inlineStr">
         <is>
           <t>1.1 Conclusão da análise crítica do certificado de calibração:</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="28" t="inlineStr">
+      <c r="A38" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">O certificado está conforme e atende ao procedimento?  </t>
         </is>
       </c>
     </row>
-    <row r="39" ht="16.5" customHeight="1" s="15">
-      <c r="A39" s="24" t="inlineStr">
+    <row r="39" ht="16.5" customHeight="1" s="19">
+      <c r="A39" s="18" t="inlineStr">
         <is>
           <t>◉ Sim  ○ Não</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="24" t="n"/>
-      <c r="B40" s="24" t="n"/>
-      <c r="C40" s="24" t="n"/>
-      <c r="D40" s="24" t="n"/>
-      <c r="E40" s="24" t="n"/>
-      <c r="F40" s="24" t="n"/>
-      <c r="G40" s="24" t="n"/>
-      <c r="H40" s="24" t="n"/>
+      <c r="A40" s="18" t="n"/>
+      <c r="B40" s="18" t="n"/>
+      <c r="C40" s="18" t="n"/>
+      <c r="D40" s="18" t="n"/>
+      <c r="E40" s="18" t="n"/>
+      <c r="F40" s="18" t="n"/>
+      <c r="G40" s="18" t="n"/>
+      <c r="H40" s="18" t="n"/>
       <c r="O40" s="6" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="35" t="inlineStr">
+      <c r="A41" s="23" t="inlineStr">
         <is>
           <t>OBSERVAÇÕES:</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="44" t="inlineStr"/>
-      <c r="B42" s="13" t="n"/>
-      <c r="C42" s="13" t="n"/>
-      <c r="D42" s="13" t="n"/>
-      <c r="E42" s="13" t="n"/>
-      <c r="F42" s="13" t="n"/>
-      <c r="G42" s="13" t="n"/>
-      <c r="H42" s="11" t="n"/>
+      <c r="A42" s="32" t="inlineStr"/>
+      <c r="B42" s="33" t="n"/>
+      <c r="C42" s="33" t="n"/>
+      <c r="D42" s="33" t="n"/>
+      <c r="E42" s="33" t="n"/>
+      <c r="F42" s="33" t="n"/>
+      <c r="G42" s="33" t="n"/>
+      <c r="H42" s="27" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="17" t="n"/>
-      <c r="B43" s="18" t="n"/>
-      <c r="C43" s="18" t="n"/>
-      <c r="D43" s="18" t="n"/>
-      <c r="E43" s="18" t="n"/>
-      <c r="F43" s="18" t="n"/>
-      <c r="G43" s="18" t="n"/>
-      <c r="H43" s="19" t="n"/>
+      <c r="A43" s="29" t="n"/>
+      <c r="B43" s="34" t="n"/>
+      <c r="C43" s="34" t="n"/>
+      <c r="D43" s="34" t="n"/>
+      <c r="E43" s="34" t="n"/>
+      <c r="F43" s="34" t="n"/>
+      <c r="G43" s="34" t="n"/>
+      <c r="H43" s="30" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="45" t="n"/>
@@ -1706,7 +1706,7 @@
       <c r="H45" s="45" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="24" t="inlineStr">
+      <c r="A46" s="18" t="inlineStr">
         <is>
           <t>_____________________________________</t>
         </is>
@@ -1715,7 +1715,7 @@
     <row r="47"/>
     <row r="48"/>
     <row r="49">
-      <c r="A49" s="28" t="inlineStr">
+      <c r="A49" s="25" t="inlineStr">
         <is>
           <t>Responsável pela Análise</t>
         </is>
@@ -1725,13 +1725,13 @@
   <mergeCells count="50">
     <mergeCell ref="A30:E30"/>
     <mergeCell ref="A34:E34"/>
+    <mergeCell ref="D13:F13"/>
     <mergeCell ref="G12:H12"/>
-    <mergeCell ref="D13:F13"/>
-    <mergeCell ref="A39:H39"/>
     <mergeCell ref="F5:H5"/>
     <mergeCell ref="A24:E24"/>
+    <mergeCell ref="A15:H15"/>
     <mergeCell ref="G2:H2"/>
-    <mergeCell ref="A15:H15"/>
+    <mergeCell ref="A39:H39"/>
     <mergeCell ref="C9:E9"/>
     <mergeCell ref="A49:H49"/>
     <mergeCell ref="A12:C12"/>
@@ -1766,10 +1766,10 @@
     <mergeCell ref="A29:E29"/>
     <mergeCell ref="A20:E20"/>
     <mergeCell ref="C5:E5"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="C1:F3"/>
     <mergeCell ref="A38:H38"/>
     <mergeCell ref="A28:E28"/>
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="C1:F3"/>
     <mergeCell ref="A19:E19"/>
     <mergeCell ref="A31:E31"/>
     <mergeCell ref="C10:E10"/>

</xml_diff>

<commit_message>
ajuste na classificação dos instrumentos geração de ac e xml
</commit_message>
<xml_diff>
--- a/TemplateAC_ORIGEM.xlsx
+++ b/TemplateAC_ORIGEM.xlsx
@@ -372,7 +372,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="89">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -483,6 +483,111 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -985,7 +1090,7 @@
     <row r="6" ht="34.5" customHeight="1" s="19">
       <c r="A6" s="31" t="inlineStr">
         <is>
-          <t>TT-SG-122104-01</t>
+          <t>PDT-SG-122104-01</t>
         </is>
       </c>
       <c r="B6" s="12" t="n"/>
@@ -1034,7 +1139,7 @@
       <c r="E8" s="27" t="n"/>
       <c r="F8" s="31" t="inlineStr">
         <is>
-          <t>[ ✔ ]Termorresistência (TE)</t>
+          <t>[ ] Termorresistência (TE)</t>
         </is>
       </c>
       <c r="G8" s="33" t="n"/>
@@ -1045,7 +1150,7 @@
       <c r="B9" s="22" t="n"/>
       <c r="C9" s="24" t="inlineStr">
         <is>
-          <t>[ ] Transmissor de pressão diferencial (PDT)</t>
+          <t>[ ✔ ] Transmissor de pressão diferencial (PDT)</t>
         </is>
       </c>
       <c r="E9" s="22" t="n"/>
@@ -1057,7 +1162,7 @@
       <c r="B10" s="30" t="n"/>
       <c r="C10" s="44" t="inlineStr">
         <is>
-          <t>[ ✔ ] Transmissor de temperatura (TT)</t>
+          <t>[ ] Transmissor de temperatura (TT)</t>
         </is>
       </c>
       <c r="D10" s="34" t="n"/>
@@ -1091,7 +1196,7 @@
     <row r="13">
       <c r="A13" s="31" t="inlineStr">
         <is>
-          <t>25-ODS-0638 - TEM - 150</t>
+          <t>25-ODS-0638 - PRE - 231</t>
         </is>
       </c>
       <c r="B13" s="11" t="n"/>
@@ -1713,18 +1818,18 @@
       <c r="H43" s="30" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="52" t="n"/>
-      <c r="B45" s="52" t="n"/>
-      <c r="C45" s="52" t="n"/>
-      <c r="D45" s="53" t="inlineStr">
+      <c r="A45" s="87" t="n"/>
+      <c r="B45" s="87" t="n"/>
+      <c r="C45" s="87" t="n"/>
+      <c r="D45" s="88" t="inlineStr">
         <is>
           <t>Data: 12/09/2025</t>
         </is>
       </c>
-      <c r="E45" s="52" t="n"/>
-      <c r="F45" s="52" t="n"/>
-      <c r="G45" s="52" t="n"/>
-      <c r="H45" s="52" t="n"/>
+      <c r="E45" s="87" t="n"/>
+      <c r="F45" s="87" t="n"/>
+      <c r="G45" s="87" t="n"/>
+      <c r="H45" s="87" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="18" t="inlineStr">

</xml_diff>

<commit_message>
inserção AC Yinson + XML somente PRIO + COMEÇO DE CRIAÇÃO XML PETROBRÁS
</commit_message>
<xml_diff>
--- a/TemplateAC_ORIGEM.xlsx
+++ b/TemplateAC_ORIGEM.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-13380" yWindow="-16320" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="15420" yWindow="-16320" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Template Formulário" sheetId="1" state="visible" r:id="rId1"/>
@@ -372,7 +372,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="89">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -399,32 +399,35 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -471,120 +474,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -1011,109 +900,109 @@
   <dimension ref="A1:O49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
-    <col width="15" customWidth="1" style="19" min="1" max="4"/>
-    <col width="11.7265625" customWidth="1" style="19" min="5" max="5"/>
-    <col width="12.453125" customWidth="1" style="19" min="6" max="6"/>
-    <col width="4.90625" bestFit="1" customWidth="1" style="19" min="7" max="7"/>
-    <col width="15" customWidth="1" style="19" min="8" max="8"/>
+    <col width="15" customWidth="1" style="21" min="1" max="4"/>
+    <col width="11.7265625" customWidth="1" style="21" min="5" max="5"/>
+    <col width="12.453125" customWidth="1" style="21" min="6" max="6"/>
+    <col width="4.90625" bestFit="1" customWidth="1" style="21" min="7" max="7"/>
+    <col width="15" customWidth="1" style="21" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20" customHeight="1" s="19">
-      <c r="A1" s="26" t="n"/>
-      <c r="B1" s="27" t="n"/>
-      <c r="C1" s="43" t="inlineStr">
+    <row r="1" ht="20" customHeight="1" s="21">
+      <c r="A1" s="27" t="n"/>
+      <c r="B1" s="28" t="n"/>
+      <c r="C1" s="44" t="inlineStr">
         <is>
           <t>REGISTRO DE ANÁLISE CRÍTICA DE CERTIFICADO DE CALIBRAÇÃO DE SECUNDÁRIOS</t>
         </is>
       </c>
-      <c r="D1" s="33" t="n"/>
-      <c r="E1" s="33" t="n"/>
-      <c r="F1" s="27" t="n"/>
-      <c r="G1" s="42" t="inlineStr">
+      <c r="D1" s="34" t="n"/>
+      <c r="E1" s="34" t="n"/>
+      <c r="F1" s="28" t="n"/>
+      <c r="G1" s="43" t="inlineStr">
         <is>
           <t>FO-COR-GER-CPROD-030</t>
         </is>
       </c>
-      <c r="H1" s="27" t="n"/>
-    </row>
-    <row r="2" ht="20" customHeight="1" s="19">
-      <c r="A2" s="28" t="n"/>
-      <c r="B2" s="22" t="n"/>
-      <c r="C2" s="28" t="n"/>
-      <c r="F2" s="22" t="n"/>
-      <c r="G2" s="21" t="inlineStr">
+      <c r="H1" s="28" t="n"/>
+    </row>
+    <row r="2" ht="20" customHeight="1" s="21">
+      <c r="A2" s="29" t="n"/>
+      <c r="B2" s="23" t="n"/>
+      <c r="C2" s="29" t="n"/>
+      <c r="F2" s="23" t="n"/>
+      <c r="G2" s="22" t="inlineStr">
         <is>
           <t>Revisão: 0</t>
         </is>
       </c>
-      <c r="H2" s="22" t="n"/>
-    </row>
-    <row r="3" ht="20" customHeight="1" s="19">
-      <c r="A3" s="29" t="n"/>
-      <c r="B3" s="30" t="n"/>
-      <c r="C3" s="29" t="n"/>
-      <c r="D3" s="34" t="n"/>
-      <c r="E3" s="34" t="n"/>
-      <c r="F3" s="30" t="n"/>
-      <c r="G3" s="40" t="inlineStr">
+      <c r="H2" s="23" t="n"/>
+    </row>
+    <row r="3" ht="20" customHeight="1" s="21">
+      <c r="A3" s="30" t="n"/>
+      <c r="B3" s="31" t="n"/>
+      <c r="C3" s="30" t="n"/>
+      <c r="D3" s="35" t="n"/>
+      <c r="E3" s="35" t="n"/>
+      <c r="F3" s="31" t="n"/>
+      <c r="G3" s="41" t="inlineStr">
         <is>
           <t>Página: 1/1</t>
         </is>
       </c>
-      <c r="H3" s="30" t="n"/>
+      <c r="H3" s="31" t="n"/>
     </row>
     <row r="4">
       <c r="G4" s="2" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="20" t="inlineStr">
+      <c r="A5" s="19" t="inlineStr">
         <is>
           <t>TAG</t>
         </is>
       </c>
-      <c r="B5" s="12" t="n"/>
-      <c r="C5" s="20" t="inlineStr">
+      <c r="B5" s="13" t="n"/>
+      <c r="C5" s="19" t="inlineStr">
         <is>
           <t>Localização</t>
         </is>
       </c>
-      <c r="D5" s="11" t="n"/>
-      <c r="E5" s="12" t="n"/>
-      <c r="F5" s="20" t="inlineStr">
+      <c r="D5" s="12" t="n"/>
+      <c r="E5" s="13" t="n"/>
+      <c r="F5" s="19" t="inlineStr">
         <is>
           <t>Identificação</t>
         </is>
       </c>
-      <c r="G5" s="11" t="n"/>
-      <c r="H5" s="12" t="n"/>
-    </row>
-    <row r="6" ht="34.5" customHeight="1" s="19">
-      <c r="A6" s="31" t="inlineStr">
+      <c r="G5" s="12" t="n"/>
+      <c r="H5" s="13" t="n"/>
+    </row>
+    <row r="6" ht="34.5" customHeight="1" s="21">
+      <c r="A6" s="32" t="inlineStr">
         <is>
           <t>PDT-SG-122104-01</t>
         </is>
       </c>
-      <c r="B6" s="12" t="n"/>
-      <c r="C6" s="31" t="inlineStr">
+      <c r="B6" s="13" t="n"/>
+      <c r="C6" s="32" t="inlineStr">
         <is>
           <t>teste</t>
         </is>
       </c>
-      <c r="D6" s="11" t="n"/>
-      <c r="E6" s="12" t="n"/>
+      <c r="D6" s="12" t="n"/>
+      <c r="E6" s="13" t="n"/>
       <c r="F6" s="8" t="inlineStr">
         <is>
           <t>SAP: teste</t>
         </is>
       </c>
-      <c r="G6" s="31" t="inlineStr">
+      <c r="G6" s="32" t="inlineStr">
         <is>
           <t>CE: teste</t>
         </is>
       </c>
-      <c r="H6" s="12" t="n"/>
-    </row>
-    <row r="7" ht="14.5" customHeight="1" s="19">
+      <c r="H6" s="13" t="n"/>
+    </row>
+    <row r="7" ht="14.5" customHeight="1" s="21">
       <c r="A7" s="2" t="n"/>
       <c r="B7" s="2" t="n"/>
       <c r="C7" s="2" t="n"/>
@@ -1123,97 +1012,97 @@
       <c r="G7" s="3" t="n"/>
       <c r="H7" s="3" t="n"/>
     </row>
-    <row r="8" ht="14.5" customHeight="1" s="19">
-      <c r="A8" s="41" t="inlineStr">
+    <row r="8" ht="14.5" customHeight="1" s="21">
+      <c r="A8" s="42" t="inlineStr">
         <is>
           <t>OUTRAS INFORMAÇÕES (Descrição):</t>
         </is>
       </c>
-      <c r="B8" s="27" t="n"/>
-      <c r="C8" s="36" t="inlineStr">
+      <c r="B8" s="28" t="n"/>
+      <c r="C8" s="37" t="inlineStr">
         <is>
           <t>[ ] Transmissor de pressão estática (PT)</t>
         </is>
       </c>
-      <c r="D8" s="33" t="n"/>
-      <c r="E8" s="27" t="n"/>
-      <c r="F8" s="31" t="inlineStr">
+      <c r="D8" s="34" t="n"/>
+      <c r="E8" s="28" t="n"/>
+      <c r="F8" s="32" t="inlineStr">
         <is>
           <t>[ ] Termorresistência (TE)</t>
         </is>
       </c>
-      <c r="G8" s="33" t="n"/>
-      <c r="H8" s="27" t="n"/>
+      <c r="G8" s="34" t="n"/>
+      <c r="H8" s="28" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="28" t="n"/>
-      <c r="B9" s="22" t="n"/>
-      <c r="C9" s="24" t="inlineStr">
+      <c r="A9" s="29" t="n"/>
+      <c r="B9" s="23" t="n"/>
+      <c r="C9" s="25" t="inlineStr">
         <is>
           <t>[ ✔ ] Transmissor de pressão diferencial (PDT)</t>
         </is>
       </c>
-      <c r="E9" s="22" t="n"/>
-      <c r="F9" s="28" t="n"/>
-      <c r="H9" s="22" t="n"/>
+      <c r="E9" s="23" t="n"/>
+      <c r="F9" s="29" t="n"/>
+      <c r="H9" s="23" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="29" t="n"/>
-      <c r="B10" s="30" t="n"/>
-      <c r="C10" s="44" t="inlineStr">
+      <c r="A10" s="30" t="n"/>
+      <c r="B10" s="31" t="n"/>
+      <c r="C10" s="45" t="inlineStr">
         <is>
           <t>[ ] Transmissor de temperatura (TT)</t>
         </is>
       </c>
-      <c r="D10" s="34" t="n"/>
-      <c r="E10" s="30" t="n"/>
-      <c r="F10" s="29" t="n"/>
-      <c r="G10" s="34" t="n"/>
-      <c r="H10" s="30" t="n"/>
+      <c r="D10" s="35" t="n"/>
+      <c r="E10" s="31" t="n"/>
+      <c r="F10" s="30" t="n"/>
+      <c r="G10" s="35" t="n"/>
+      <c r="H10" s="31" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="20" t="inlineStr">
+      <c r="A12" s="19" t="inlineStr">
         <is>
           <t>Nº do Certificado</t>
         </is>
       </c>
-      <c r="B12" s="11" t="n"/>
-      <c r="C12" s="12" t="n"/>
-      <c r="D12" s="37" t="inlineStr">
+      <c r="B12" s="12" t="n"/>
+      <c r="C12" s="13" t="n"/>
+      <c r="D12" s="38" t="inlineStr">
         <is>
           <t>Data da Calibração</t>
         </is>
       </c>
-      <c r="E12" s="38" t="n"/>
-      <c r="F12" s="14" t="n"/>
-      <c r="G12" s="13" t="inlineStr">
+      <c r="E12" s="39" t="n"/>
+      <c r="F12" s="18" t="n"/>
+      <c r="G12" s="17" t="inlineStr">
         <is>
           <t>Empresa Certificadora</t>
         </is>
       </c>
-      <c r="H12" s="14" t="n"/>
+      <c r="H12" s="18" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="31" t="inlineStr">
+      <c r="A13" s="32" t="inlineStr">
         <is>
           <t>25-ODS-0638 - PRE - 231</t>
         </is>
       </c>
-      <c r="B13" s="11" t="n"/>
-      <c r="C13" s="12" t="n"/>
-      <c r="D13" s="15" t="inlineStr">
+      <c r="B13" s="12" t="n"/>
+      <c r="C13" s="13" t="n"/>
+      <c r="D13" s="14" t="inlineStr">
         <is>
           <t>01/09/2025</t>
         </is>
       </c>
-      <c r="E13" s="16" t="n"/>
-      <c r="F13" s="17" t="n"/>
-      <c r="G13" s="39" t="inlineStr">
+      <c r="E13" s="15" t="n"/>
+      <c r="F13" s="16" t="n"/>
+      <c r="G13" s="40" t="inlineStr">
         <is>
           <t>ODS Lab</t>
         </is>
       </c>
-      <c r="H13" s="17" t="n"/>
+      <c r="H13" s="16" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n"/>
@@ -1226,48 +1115,48 @@
       <c r="H14" s="2" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="23" t="inlineStr">
+      <c r="A15" s="20" t="inlineStr">
         <is>
           <t>1 - ANÁLISE DO CERTIFICADO DE CALIBRAÇÃO</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="25" customHeight="1" s="19">
-      <c r="A16" s="35" t="inlineStr">
+    <row r="16" ht="25" customHeight="1" s="21">
+      <c r="A16" s="36" t="inlineStr">
         <is>
           <t>DESCRIÇÃO DOS ITENS A SEREM VERIFICADOS</t>
         </is>
       </c>
-      <c r="B16" s="11" t="n"/>
-      <c r="C16" s="11" t="n"/>
-      <c r="D16" s="11" t="n"/>
-      <c r="E16" s="12" t="n"/>
-      <c r="F16" s="35" t="inlineStr">
+      <c r="B16" s="12" t="n"/>
+      <c r="C16" s="12" t="n"/>
+      <c r="D16" s="12" t="n"/>
+      <c r="E16" s="13" t="n"/>
+      <c r="F16" s="36" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
       </c>
-      <c r="G16" s="35" t="inlineStr">
+      <c r="G16" s="36" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
-      <c r="H16" s="35" t="inlineStr">
+      <c r="H16" s="36" t="inlineStr">
         <is>
           <t>NÃO APLICÁVEL</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="16.5" customHeight="1" s="19">
-      <c r="A17" s="10" t="inlineStr">
+    <row r="17" ht="16.5" customHeight="1" s="21">
+      <c r="A17" s="11" t="inlineStr">
         <is>
           <t>a) Identificação unívoca (Número do Certificado de Calibração).</t>
         </is>
       </c>
-      <c r="B17" s="11" t="n"/>
-      <c r="C17" s="11" t="n"/>
-      <c r="D17" s="11" t="n"/>
-      <c r="E17" s="12" t="n"/>
+      <c r="B17" s="12" t="n"/>
+      <c r="C17" s="12" t="n"/>
+      <c r="D17" s="12" t="n"/>
+      <c r="E17" s="13" t="n"/>
       <c r="F17" s="7" t="inlineStr">
         <is>
           <t>◉</t>
@@ -1284,16 +1173,16 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="16.5" customHeight="1" s="19">
-      <c r="A18" s="10" t="inlineStr">
+    <row r="18" ht="16.5" customHeight="1" s="21">
+      <c r="A18" s="11" t="inlineStr">
         <is>
           <t>b) Nome e endereço do Laboratório/Empresa.</t>
         </is>
       </c>
-      <c r="B18" s="11" t="n"/>
-      <c r="C18" s="11" t="n"/>
-      <c r="D18" s="11" t="n"/>
-      <c r="E18" s="12" t="n"/>
+      <c r="B18" s="12" t="n"/>
+      <c r="C18" s="12" t="n"/>
+      <c r="D18" s="12" t="n"/>
+      <c r="E18" s="13" t="n"/>
       <c r="F18" s="7" t="inlineStr">
         <is>
           <t>◉</t>
@@ -1310,16 +1199,16 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="31" customHeight="1" s="19">
-      <c r="A19" s="10" t="inlineStr">
+    <row r="19" ht="31" customHeight="1" s="21">
+      <c r="A19" s="11" t="inlineStr">
         <is>
           <t>c) Logotipo da RBC (para instrumento associado a sistemas de medição fiscal, apropriação, custódia, flare)</t>
         </is>
       </c>
-      <c r="B19" s="11" t="n"/>
-      <c r="C19" s="11" t="n"/>
-      <c r="D19" s="11" t="n"/>
-      <c r="E19" s="12" t="n"/>
+      <c r="B19" s="12" t="n"/>
+      <c r="C19" s="12" t="n"/>
+      <c r="D19" s="12" t="n"/>
+      <c r="E19" s="13" t="n"/>
       <c r="F19" s="7" t="inlineStr">
         <is>
           <t>◉</t>
@@ -1336,16 +1225,16 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="16.5" customHeight="1" s="19">
-      <c r="A20" s="10" t="inlineStr">
+    <row r="20" ht="16.5" customHeight="1" s="21">
+      <c r="A20" s="11" t="inlineStr">
         <is>
           <t>d) Nome e endereço do cliente.</t>
         </is>
       </c>
-      <c r="B20" s="11" t="n"/>
-      <c r="C20" s="11" t="n"/>
-      <c r="D20" s="11" t="n"/>
-      <c r="E20" s="12" t="n"/>
+      <c r="B20" s="12" t="n"/>
+      <c r="C20" s="12" t="n"/>
+      <c r="D20" s="12" t="n"/>
+      <c r="E20" s="13" t="n"/>
       <c r="F20" s="7" t="inlineStr">
         <is>
           <t>◉</t>
@@ -1362,16 +1251,16 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="16.5" customHeight="1" s="19">
-      <c r="A21" s="10" t="inlineStr">
+    <row r="21" ht="16.5" customHeight="1" s="21">
+      <c r="A21" s="11" t="inlineStr">
         <is>
           <t>e) Número de páginas e total de páginas.</t>
         </is>
       </c>
-      <c r="B21" s="11" t="n"/>
-      <c r="C21" s="11" t="n"/>
-      <c r="D21" s="11" t="n"/>
-      <c r="E21" s="12" t="n"/>
+      <c r="B21" s="12" t="n"/>
+      <c r="C21" s="12" t="n"/>
+      <c r="D21" s="12" t="n"/>
+      <c r="E21" s="13" t="n"/>
       <c r="F21" s="7" t="inlineStr">
         <is>
           <t>◉</t>
@@ -1388,16 +1277,16 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="16.5" customHeight="1" s="19">
-      <c r="A22" s="10" t="inlineStr">
+    <row r="22" ht="16.5" customHeight="1" s="21">
+      <c r="A22" s="11" t="inlineStr">
         <is>
           <t>f) Identificação do método/procedimento utilizado.</t>
         </is>
       </c>
-      <c r="B22" s="11" t="n"/>
-      <c r="C22" s="11" t="n"/>
-      <c r="D22" s="11" t="n"/>
-      <c r="E22" s="12" t="n"/>
+      <c r="B22" s="12" t="n"/>
+      <c r="C22" s="12" t="n"/>
+      <c r="D22" s="12" t="n"/>
+      <c r="E22" s="13" t="n"/>
       <c r="F22" s="7" t="inlineStr">
         <is>
           <t>◉</t>
@@ -1414,16 +1303,16 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="16.5" customHeight="1" s="19">
-      <c r="A23" s="10" t="inlineStr">
+    <row r="23" ht="16.5" customHeight="1" s="21">
+      <c r="A23" s="11" t="inlineStr">
         <is>
           <t>g) Registro das condições ambientais.</t>
         </is>
       </c>
-      <c r="B23" s="11" t="n"/>
-      <c r="C23" s="11" t="n"/>
-      <c r="D23" s="11" t="n"/>
-      <c r="E23" s="12" t="n"/>
+      <c r="B23" s="12" t="n"/>
+      <c r="C23" s="12" t="n"/>
+      <c r="D23" s="12" t="n"/>
+      <c r="E23" s="13" t="n"/>
       <c r="F23" s="7" t="inlineStr">
         <is>
           <t>◉</t>
@@ -1440,16 +1329,16 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="31" customHeight="1" s="19">
-      <c r="A24" s="10" t="inlineStr">
+    <row r="24" ht="31" customHeight="1" s="21">
+      <c r="A24" s="11" t="inlineStr">
         <is>
           <t>h) Descrição e identificação do item de calibração (ex.: nome, fabricante, tipo, modelo, número de série, outra identificação estabelecida pelo cliente).</t>
         </is>
       </c>
-      <c r="B24" s="11" t="n"/>
-      <c r="C24" s="11" t="n"/>
-      <c r="D24" s="11" t="n"/>
-      <c r="E24" s="12" t="n"/>
+      <c r="B24" s="12" t="n"/>
+      <c r="C24" s="12" t="n"/>
+      <c r="D24" s="12" t="n"/>
+      <c r="E24" s="13" t="n"/>
       <c r="F24" s="7" t="inlineStr">
         <is>
           <t>◉</t>
@@ -1466,16 +1355,16 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="16.5" customHeight="1" s="19">
-      <c r="A25" s="10" t="inlineStr">
+    <row r="25" ht="16.5" customHeight="1" s="21">
+      <c r="A25" s="11" t="inlineStr">
         <is>
           <t>i) A data do recebimento do(s) item(s) de calibração, se necessário.</t>
         </is>
       </c>
-      <c r="B25" s="11" t="n"/>
-      <c r="C25" s="11" t="n"/>
-      <c r="D25" s="11" t="n"/>
-      <c r="E25" s="12" t="n"/>
+      <c r="B25" s="12" t="n"/>
+      <c r="C25" s="12" t="n"/>
+      <c r="D25" s="12" t="n"/>
+      <c r="E25" s="13" t="n"/>
       <c r="F25" s="7" t="inlineStr">
         <is>
           <t>○</t>
@@ -1492,16 +1381,16 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="16.5" customHeight="1" s="19">
-      <c r="A26" s="10" t="inlineStr">
+    <row r="26" ht="16.5" customHeight="1" s="21">
+      <c r="A26" s="11" t="inlineStr">
         <is>
           <t>j) A data da realização da calibração.</t>
         </is>
       </c>
-      <c r="B26" s="11" t="n"/>
-      <c r="C26" s="11" t="n"/>
-      <c r="D26" s="11" t="n"/>
-      <c r="E26" s="12" t="n"/>
+      <c r="B26" s="12" t="n"/>
+      <c r="C26" s="12" t="n"/>
+      <c r="D26" s="12" t="n"/>
+      <c r="E26" s="13" t="n"/>
       <c r="F26" s="7" t="inlineStr">
         <is>
           <t>◉</t>
@@ -1518,16 +1407,16 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="31" customHeight="1" s="19">
-      <c r="A27" s="10" t="inlineStr">
+    <row r="27" ht="31" customHeight="1" s="21">
+      <c r="A27" s="11" t="inlineStr">
         <is>
           <t>k) Os resultados da calibração estão com as unidades de medida no SI, onde apropriado.</t>
         </is>
       </c>
-      <c r="B27" s="11" t="n"/>
-      <c r="C27" s="11" t="n"/>
-      <c r="D27" s="11" t="n"/>
-      <c r="E27" s="12" t="n"/>
+      <c r="B27" s="12" t="n"/>
+      <c r="C27" s="12" t="n"/>
+      <c r="D27" s="12" t="n"/>
+      <c r="E27" s="13" t="n"/>
       <c r="F27" s="7" t="inlineStr">
         <is>
           <t>◉</t>
@@ -1544,16 +1433,16 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="16.5" customHeight="1" s="19">
-      <c r="A28" s="10" t="inlineStr">
+    <row r="28" ht="16.5" customHeight="1" s="21">
+      <c r="A28" s="11" t="inlineStr">
         <is>
           <t>l) Evidências de que as medições são rastreáveis (Informações dos padrões utilizados).</t>
         </is>
       </c>
-      <c r="B28" s="11" t="n"/>
-      <c r="C28" s="11" t="n"/>
-      <c r="D28" s="11" t="n"/>
-      <c r="E28" s="12" t="n"/>
+      <c r="B28" s="12" t="n"/>
+      <c r="C28" s="12" t="n"/>
+      <c r="D28" s="12" t="n"/>
+      <c r="E28" s="13" t="n"/>
       <c r="F28" s="7" t="inlineStr">
         <is>
           <t>◉</t>
@@ -1570,16 +1459,16 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="31" customHeight="1" s="19">
-      <c r="A29" s="10" t="inlineStr">
+    <row r="29" ht="31" customHeight="1" s="21">
+      <c r="A29" s="11" t="inlineStr">
         <is>
           <t>m) Nome(s), função (ões) e assinatura (s) ou identificações equivalentes das pessoas autorizadas para emissão do certificado.</t>
         </is>
       </c>
-      <c r="B29" s="11" t="n"/>
-      <c r="C29" s="11" t="n"/>
-      <c r="D29" s="11" t="n"/>
-      <c r="E29" s="12" t="n"/>
+      <c r="B29" s="12" t="n"/>
+      <c r="C29" s="12" t="n"/>
+      <c r="D29" s="12" t="n"/>
+      <c r="E29" s="13" t="n"/>
       <c r="F29" s="7" t="inlineStr">
         <is>
           <t>◉</t>
@@ -1596,16 +1485,16 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="31" customHeight="1" s="19">
-      <c r="A30" s="10" t="inlineStr">
+    <row r="30" ht="31" customHeight="1" s="21">
+      <c r="A30" s="11" t="inlineStr">
         <is>
           <t>n) Declaração de que os resultados e incertezas se referem somente aos itens calibrados / inspecionados.</t>
         </is>
       </c>
-      <c r="B30" s="11" t="n"/>
-      <c r="C30" s="11" t="n"/>
-      <c r="D30" s="11" t="n"/>
-      <c r="E30" s="12" t="n"/>
+      <c r="B30" s="12" t="n"/>
+      <c r="C30" s="12" t="n"/>
+      <c r="D30" s="12" t="n"/>
+      <c r="E30" s="13" t="n"/>
       <c r="F30" s="7" t="inlineStr">
         <is>
           <t>◉</t>
@@ -1622,16 +1511,16 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="16.5" customHeight="1" s="19">
-      <c r="A31" s="10" t="inlineStr">
+    <row r="31" ht="16.5" customHeight="1" s="21">
+      <c r="A31" s="11" t="inlineStr">
         <is>
           <t>o) Nível de confiança e fator de abrangência.</t>
         </is>
       </c>
-      <c r="B31" s="11" t="n"/>
-      <c r="C31" s="11" t="n"/>
-      <c r="D31" s="11" t="n"/>
-      <c r="E31" s="12" t="n"/>
+      <c r="B31" s="12" t="n"/>
+      <c r="C31" s="12" t="n"/>
+      <c r="D31" s="12" t="n"/>
+      <c r="E31" s="13" t="n"/>
       <c r="F31" s="7" t="inlineStr">
         <is>
           <t>◉</t>
@@ -1648,16 +1537,16 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="16.5" customHeight="1" s="19">
-      <c r="A32" s="10" t="inlineStr">
+    <row r="32" ht="16.5" customHeight="1" s="21">
+      <c r="A32" s="11" t="inlineStr">
         <is>
           <t>p) Foi feita calibração de acordo com a faixa solicitada?</t>
         </is>
       </c>
-      <c r="B32" s="11" t="n"/>
-      <c r="C32" s="11" t="n"/>
-      <c r="D32" s="11" t="n"/>
-      <c r="E32" s="12" t="n"/>
+      <c r="B32" s="12" t="n"/>
+      <c r="C32" s="12" t="n"/>
+      <c r="D32" s="12" t="n"/>
+      <c r="E32" s="13" t="n"/>
       <c r="F32" s="7" t="inlineStr">
         <is>
           <t>◉</t>
@@ -1674,16 +1563,16 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="31" customHeight="1" s="19">
-      <c r="A33" s="10" t="inlineStr">
+    <row r="33" ht="31" customHeight="1" s="21">
+      <c r="A33" s="11" t="inlineStr">
         <is>
           <t>q) Os erros máximos de medição (Erro sistemático remanescente + incerteza) são inferiores ao erro máximo admissível para o equipamento em questão?</t>
         </is>
       </c>
-      <c r="B33" s="11" t="n"/>
-      <c r="C33" s="11" t="n"/>
-      <c r="D33" s="11" t="n"/>
-      <c r="E33" s="12" t="n"/>
+      <c r="B33" s="12" t="n"/>
+      <c r="C33" s="12" t="n"/>
+      <c r="D33" s="12" t="n"/>
+      <c r="E33" s="13" t="n"/>
       <c r="F33" s="7" t="inlineStr">
         <is>
           <t>◉</t>
@@ -1700,16 +1589,16 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="31" customHeight="1" s="19">
-      <c r="A34" s="10" t="inlineStr">
+    <row r="34" ht="31" customHeight="1" s="21">
+      <c r="A34" s="11" t="inlineStr">
         <is>
           <t>r) O instrumento está aprovado para o uso no ponto de medição a que se destina de acordo com os critérios de aceitação informados pelo cliente?</t>
         </is>
       </c>
-      <c r="B34" s="11" t="n"/>
-      <c r="C34" s="11" t="n"/>
-      <c r="D34" s="11" t="n"/>
-      <c r="E34" s="12" t="n"/>
+      <c r="B34" s="12" t="n"/>
+      <c r="C34" s="12" t="n"/>
+      <c r="D34" s="12" t="n"/>
+      <c r="E34" s="13" t="n"/>
       <c r="F34" s="7" t="inlineStr">
         <is>
           <t>◉</t>
@@ -1726,22 +1615,22 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="31" customHeight="1" s="19">
-      <c r="A35" s="10" t="inlineStr">
+    <row r="35" ht="31" customHeight="1" s="21">
+      <c r="A35" s="11" t="inlineStr">
         <is>
           <t>s) No caso de ajuste no equipamento, estão informados os resultados das calibrações como encontrados (as found) e como deixados (as left)?</t>
         </is>
       </c>
-      <c r="B35" s="11" t="n"/>
-      <c r="C35" s="11" t="n"/>
-      <c r="D35" s="11" t="n"/>
-      <c r="E35" s="12" t="n"/>
+      <c r="B35" s="12" t="n"/>
+      <c r="C35" s="12" t="n"/>
+      <c r="D35" s="12" t="n"/>
+      <c r="E35" s="13" t="n"/>
       <c r="F35" s="7" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="G35" s="48" t="inlineStr">
+      <c r="G35" s="10" t="inlineStr">
         <is>
           <t>●</t>
         </is>
@@ -1759,80 +1648,80 @@
       <c r="H36" s="2" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="23" t="inlineStr">
+      <c r="A37" s="20" t="inlineStr">
         <is>
           <t>1.1 Conclusão da análise crítica do certificado de calibração:</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="25" t="inlineStr">
+      <c r="A38" s="26" t="inlineStr">
         <is>
           <t xml:space="preserve">O certificado está conforme e atende ao procedimento?  </t>
         </is>
       </c>
     </row>
-    <row r="39" ht="16.5" customHeight="1" s="19">
-      <c r="A39" s="18" t="inlineStr">
+    <row r="39" ht="16.5" customHeight="1" s="21">
+      <c r="A39" s="24" t="inlineStr">
         <is>
           <t>◉ Sim  ○ Não</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="18" t="n"/>
-      <c r="B40" s="18" t="n"/>
-      <c r="C40" s="18" t="n"/>
-      <c r="D40" s="18" t="n"/>
-      <c r="E40" s="18" t="n"/>
-      <c r="F40" s="18" t="n"/>
-      <c r="G40" s="18" t="n"/>
-      <c r="H40" s="18" t="n"/>
+      <c r="A40" s="24" t="n"/>
+      <c r="B40" s="24" t="n"/>
+      <c r="C40" s="24" t="n"/>
+      <c r="D40" s="24" t="n"/>
+      <c r="E40" s="24" t="n"/>
+      <c r="F40" s="24" t="n"/>
+      <c r="G40" s="24" t="n"/>
+      <c r="H40" s="24" t="n"/>
       <c r="O40" s="6" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="23" t="inlineStr">
+      <c r="A41" s="20" t="inlineStr">
         <is>
           <t>OBSERVAÇÕES:</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="32" t="inlineStr"/>
-      <c r="B42" s="33" t="n"/>
-      <c r="C42" s="33" t="n"/>
-      <c r="D42" s="33" t="n"/>
-      <c r="E42" s="33" t="n"/>
-      <c r="F42" s="33" t="n"/>
-      <c r="G42" s="33" t="n"/>
-      <c r="H42" s="27" t="n"/>
+      <c r="A42" s="33" t="inlineStr"/>
+      <c r="B42" s="34" t="n"/>
+      <c r="C42" s="34" t="n"/>
+      <c r="D42" s="34" t="n"/>
+      <c r="E42" s="34" t="n"/>
+      <c r="F42" s="34" t="n"/>
+      <c r="G42" s="34" t="n"/>
+      <c r="H42" s="28" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="29" t="n"/>
-      <c r="B43" s="34" t="n"/>
-      <c r="C43" s="34" t="n"/>
-      <c r="D43" s="34" t="n"/>
-      <c r="E43" s="34" t="n"/>
-      <c r="F43" s="34" t="n"/>
-      <c r="G43" s="34" t="n"/>
-      <c r="H43" s="30" t="n"/>
+      <c r="A43" s="30" t="n"/>
+      <c r="B43" s="35" t="n"/>
+      <c r="C43" s="35" t="n"/>
+      <c r="D43" s="35" t="n"/>
+      <c r="E43" s="35" t="n"/>
+      <c r="F43" s="35" t="n"/>
+      <c r="G43" s="35" t="n"/>
+      <c r="H43" s="31" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="87" t="n"/>
-      <c r="B45" s="87" t="n"/>
-      <c r="C45" s="87" t="n"/>
-      <c r="D45" s="88" t="inlineStr">
+      <c r="A45" s="50" t="n"/>
+      <c r="B45" s="50" t="n"/>
+      <c r="C45" s="50" t="n"/>
+      <c r="D45" s="51" t="inlineStr">
         <is>
           <t>Data: 12/09/2025</t>
         </is>
       </c>
-      <c r="E45" s="87" t="n"/>
-      <c r="F45" s="87" t="n"/>
-      <c r="G45" s="87" t="n"/>
-      <c r="H45" s="87" t="n"/>
+      <c r="E45" s="50" t="n"/>
+      <c r="F45" s="50" t="n"/>
+      <c r="G45" s="50" t="n"/>
+      <c r="H45" s="50" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="18" t="inlineStr">
+      <c r="A46" s="24" t="inlineStr">
         <is>
           <t>_____________________________________</t>
         </is>
@@ -1841,7 +1730,7 @@
     <row r="47"/>
     <row r="48"/>
     <row r="49">
-      <c r="A49" s="25" t="inlineStr">
+      <c r="A49" s="26" t="inlineStr">
         <is>
           <t>Responsável pela Análise</t>
         </is>
@@ -1851,13 +1740,13 @@
   <mergeCells count="50">
     <mergeCell ref="A30:E30"/>
     <mergeCell ref="A34:E34"/>
+    <mergeCell ref="G12:H12"/>
     <mergeCell ref="D13:F13"/>
-    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="A39:H39"/>
     <mergeCell ref="F5:H5"/>
     <mergeCell ref="A24:E24"/>
+    <mergeCell ref="G2:H2"/>
     <mergeCell ref="A15:H15"/>
-    <mergeCell ref="G2:H2"/>
-    <mergeCell ref="A39:H39"/>
     <mergeCell ref="C9:E9"/>
     <mergeCell ref="A49:H49"/>
     <mergeCell ref="A12:C12"/>
@@ -1892,16 +1781,16 @@
     <mergeCell ref="A29:E29"/>
     <mergeCell ref="A20:E20"/>
     <mergeCell ref="C5:E5"/>
+    <mergeCell ref="A38:H38"/>
+    <mergeCell ref="A28:E28"/>
     <mergeCell ref="G1:H1"/>
     <mergeCell ref="C1:F3"/>
-    <mergeCell ref="A38:H38"/>
-    <mergeCell ref="A28:E28"/>
     <mergeCell ref="A19:E19"/>
     <mergeCell ref="A31:E31"/>
     <mergeCell ref="C10:E10"/>
   </mergeCells>
   <pageMargins left="0.8" right="0.5" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" scale="73" fitToHeight="1" fitToWidth="1"/>
+  <pageSetup orientation="portrait" scale="77" fitToHeight="1" fitToWidth="1"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fluxo placa e xml inclusos
</commit_message>
<xml_diff>
--- a/TemplateAC_ORIGEM.xlsx
+++ b/TemplateAC_ORIGEM.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="15420" yWindow="-16320" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Template Formulário" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template Formulário" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Template Formulário'!$A$1:$H$50</definedName>
@@ -372,7 +372,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -474,6 +474,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -570,7 +573,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -585,20 +588,20 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:xfrm>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:off x="285750" y="142875"/>
           <a:ext cx="1428750" cy="476250"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
           <avLst/>
         </a:prstGeom>
-        <a:ln>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
@@ -979,13 +982,13 @@
     <row r="6" ht="34.5" customHeight="1" s="21">
       <c r="A6" s="32" t="inlineStr">
         <is>
-          <t>PDT-SG-122104-01</t>
+          <t>PT-SG-122104-01</t>
         </is>
       </c>
       <c r="B6" s="13" t="n"/>
       <c r="C6" s="32" t="inlineStr">
         <is>
-          <t>teste</t>
+          <t>testet</t>
         </is>
       </c>
       <c r="D6" s="12" t="n"/>
@@ -1021,7 +1024,7 @@
       <c r="B8" s="28" t="n"/>
       <c r="C8" s="37" t="inlineStr">
         <is>
-          <t>[ ] Transmissor de pressão estática (PT)</t>
+          <t>[ ✔ ] Transmissor de pressão estática (PT)</t>
         </is>
       </c>
       <c r="D8" s="34" t="n"/>
@@ -1039,7 +1042,7 @@
       <c r="B9" s="23" t="n"/>
       <c r="C9" s="25" t="inlineStr">
         <is>
-          <t>[ ✔ ] Transmissor de pressão diferencial (PDT)</t>
+          <t>[ ] Transmissor de pressão diferencial (PDT)</t>
         </is>
       </c>
       <c r="E9" s="23" t="n"/>
@@ -1085,7 +1088,7 @@
     <row r="13">
       <c r="A13" s="32" t="inlineStr">
         <is>
-          <t>25-ODS-0638 - PRE - 231</t>
+          <t>25-ODS-0638 - PRE - 230</t>
         </is>
       </c>
       <c r="B13" s="12" t="n"/>
@@ -1707,18 +1710,18 @@
       <c r="H43" s="31" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="50" t="n"/>
-      <c r="B45" s="50" t="n"/>
-      <c r="C45" s="50" t="n"/>
-      <c r="D45" s="51" t="inlineStr">
+      <c r="A45" s="51" t="n"/>
+      <c r="B45" s="51" t="n"/>
+      <c r="C45" s="51" t="n"/>
+      <c r="D45" s="52" t="inlineStr">
         <is>
           <t>Data: 12/09/2025</t>
         </is>
       </c>
-      <c r="E45" s="50" t="n"/>
-      <c r="F45" s="50" t="n"/>
-      <c r="G45" s="50" t="n"/>
-      <c r="H45" s="50" t="n"/>
+      <c r="E45" s="51" t="n"/>
+      <c r="F45" s="51" t="n"/>
+      <c r="G45" s="51" t="n"/>
+      <c r="H45" s="51" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="24" t="inlineStr">

</xml_diff>

<commit_message>
Geração de xml petrobrás de secundários da origem ativada
</commit_message>
<xml_diff>
--- a/TemplateAC_ORIGEM.xlsx
+++ b/TemplateAC_ORIGEM.xlsx
@@ -372,7 +372,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -474,6 +474,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -964,25 +973,25 @@
     <row r="6" ht="34.5" customHeight="1" s="20">
       <c r="A6" s="32" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>TT-V-122103-01</t>
         </is>
       </c>
       <c r="B6" s="13" t="n"/>
       <c r="C6" s="32" t="inlineStr">
         <is>
-          <t>teste</t>
+          <t>TESTE</t>
         </is>
       </c>
       <c r="D6" s="12" t="n"/>
       <c r="E6" s="13" t="n"/>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>SAP: teste</t>
+          <t>SAP: TESTE</t>
         </is>
       </c>
       <c r="G6" s="32" t="inlineStr">
         <is>
-          <t>CE: teste</t>
+          <t>CE: TESTE</t>
         </is>
       </c>
       <c r="H6" s="13" t="n"/>
@@ -1006,7 +1015,7 @@
       <c r="B8" s="28" t="n"/>
       <c r="C8" s="37" t="inlineStr">
         <is>
-          <t>[ ✔ ] Transmissor de pressão estática (PT)</t>
+          <t>[ ] Transmissor de pressão estática (PT)</t>
         </is>
       </c>
       <c r="D8" s="34" t="n"/>
@@ -1036,7 +1045,7 @@
       <c r="B10" s="31" t="n"/>
       <c r="C10" s="45" t="inlineStr">
         <is>
-          <t>[ ] Transmissor de temperatura (TT)</t>
+          <t>[ ✔ ] Transmissor de temperatura (TT)</t>
         </is>
       </c>
       <c r="D10" s="35" t="n"/>
@@ -1070,12 +1079,16 @@
     <row r="13">
       <c r="A13" s="32" t="inlineStr">
         <is>
-          <t>25-ODS-0638-DIM-055</t>
+          <t>CE‐1400.0000‐6252‐811‐O2C‐013</t>
         </is>
       </c>
       <c r="B13" s="12" t="n"/>
       <c r="C13" s="13" t="n"/>
-      <c r="D13" s="16" t="n"/>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>18/03/2024</t>
+        </is>
+      </c>
       <c r="E13" s="17" t="n"/>
       <c r="F13" s="18" t="n"/>
       <c r="G13" s="40" t="inlineStr">
@@ -1688,18 +1701,18 @@
       <c r="H43" s="31" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="9" t="n"/>
-      <c r="B45" s="9" t="n"/>
-      <c r="C45" s="9" t="n"/>
-      <c r="D45" s="46" t="inlineStr">
-        <is>
-          <t>Data: 14/10/2025</t>
-        </is>
-      </c>
-      <c r="E45" s="9" t="n"/>
-      <c r="F45" s="9" t="n"/>
-      <c r="G45" s="9" t="n"/>
-      <c r="H45" s="9" t="n"/>
+      <c r="A45" s="48" t="n"/>
+      <c r="B45" s="48" t="n"/>
+      <c r="C45" s="48" t="n"/>
+      <c r="D45" s="49" t="inlineStr">
+        <is>
+          <t>Data: 20/03/2024</t>
+        </is>
+      </c>
+      <c r="E45" s="48" t="n"/>
+      <c r="F45" s="48" t="n"/>
+      <c r="G45" s="48" t="n"/>
+      <c r="H45" s="48" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="19" t="inlineStr">

</xml_diff>

<commit_message>
ajuste xml para certificados de pressão com a ajuste de calibração
</commit_message>
<xml_diff>
--- a/TemplateAC_ORIGEM.xlsx
+++ b/TemplateAC_ORIGEM.xlsx
@@ -372,7 +372,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -474,6 +474,18 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -973,25 +985,25 @@
     <row r="6" ht="34.5" customHeight="1" s="20">
       <c r="A6" s="32" t="inlineStr">
         <is>
-          <t>TT-V-122103-01</t>
+          <t>UT-SG-122101-01</t>
         </is>
       </c>
       <c r="B6" s="13" t="n"/>
       <c r="C6" s="32" t="inlineStr">
         <is>
-          <t>TESTE</t>
+          <t>teste</t>
         </is>
       </c>
       <c r="D6" s="12" t="n"/>
       <c r="E6" s="13" t="n"/>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>SAP: TESTE</t>
+          <t>SAP: teste</t>
         </is>
       </c>
       <c r="G6" s="32" t="inlineStr">
         <is>
-          <t>CE: TESTE</t>
+          <t>CE: teste</t>
         </is>
       </c>
       <c r="H6" s="13" t="n"/>
@@ -1033,7 +1045,7 @@
       <c r="B9" s="23" t="n"/>
       <c r="C9" s="25" t="inlineStr">
         <is>
-          <t>[ ] Transmissor de pressão diferencial (PDT)</t>
+          <t>[ ✔ ] Transmissor de pressão diferencial (PDT)</t>
         </is>
       </c>
       <c r="E9" s="23" t="n"/>
@@ -1045,7 +1057,7 @@
       <c r="B10" s="31" t="n"/>
       <c r="C10" s="45" t="inlineStr">
         <is>
-          <t>[ ✔ ] Transmissor de temperatura (TT)</t>
+          <t>[ ] Transmissor de temperatura (TT)</t>
         </is>
       </c>
       <c r="D10" s="35" t="n"/>
@@ -1079,14 +1091,14 @@
     <row r="13">
       <c r="A13" s="32" t="inlineStr">
         <is>
-          <t>CE‐1400.0000‐6252‐811‐O2C‐013</t>
+          <t>26-ODS-0638-PRE-444</t>
         </is>
       </c>
       <c r="B13" s="12" t="n"/>
       <c r="C13" s="13" t="n"/>
       <c r="D13" s="16" t="inlineStr">
         <is>
-          <t>18/03/2024</t>
+          <t>09/04/2026</t>
         </is>
       </c>
       <c r="E13" s="17" t="n"/>
@@ -1701,18 +1713,18 @@
       <c r="H43" s="31" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="48" t="n"/>
-      <c r="B45" s="48" t="n"/>
-      <c r="C45" s="48" t="n"/>
-      <c r="D45" s="49" t="inlineStr">
-        <is>
-          <t>Data: 20/03/2024</t>
-        </is>
-      </c>
-      <c r="E45" s="48" t="n"/>
-      <c r="F45" s="48" t="n"/>
-      <c r="G45" s="48" t="n"/>
-      <c r="H45" s="48" t="n"/>
+      <c r="A45" s="52" t="n"/>
+      <c r="B45" s="52" t="n"/>
+      <c r="C45" s="52" t="n"/>
+      <c r="D45" s="53" t="inlineStr">
+        <is>
+          <t>Data: 15/04/2026</t>
+        </is>
+      </c>
+      <c r="E45" s="52" t="n"/>
+      <c r="F45" s="52" t="n"/>
+      <c r="G45" s="52" t="n"/>
+      <c r="H45" s="52" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="19" t="inlineStr">

</xml_diff>

<commit_message>
ajuste no preenchimento da AC ORIGEM para instrumento com ajuste
</commit_message>
<xml_diff>
--- a/TemplateAC_ORIGEM.xlsx
+++ b/TemplateAC_ORIGEM.xlsx
@@ -372,7 +372,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -495,6 +495,27 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -991,19 +1012,19 @@
       <c r="B6" s="13" t="n"/>
       <c r="C6" s="32" t="inlineStr">
         <is>
-          <t>teste</t>
+          <t>TESTE</t>
         </is>
       </c>
       <c r="D6" s="12" t="n"/>
       <c r="E6" s="13" t="n"/>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>SAP: teste</t>
+          <t>SAP: TESTE</t>
         </is>
       </c>
       <c r="G6" s="32" t="inlineStr">
         <is>
-          <t>CE: teste</t>
+          <t>CE: TESTE</t>
         </is>
       </c>
       <c r="H6" s="13" t="n"/>
@@ -1631,9 +1652,9 @@
       <c r="C35" s="12" t="n"/>
       <c r="D35" s="12" t="n"/>
       <c r="E35" s="13" t="n"/>
-      <c r="F35" s="7" t="inlineStr">
-        <is>
-          <t>○</t>
+      <c r="F35" s="59" t="inlineStr">
+        <is>
+          <t>◉</t>
         </is>
       </c>
       <c r="G35" s="10" t="inlineStr">
@@ -1641,9 +1662,9 @@
           <t>●</t>
         </is>
       </c>
-      <c r="H35" s="7" t="inlineStr">
-        <is>
-          <t>◉</t>
+      <c r="H35" s="59" t="inlineStr">
+        <is>
+          <t>○</t>
         </is>
       </c>
     </row>
@@ -1713,18 +1734,18 @@
       <c r="H43" s="31" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="52" t="n"/>
-      <c r="B45" s="52" t="n"/>
-      <c r="C45" s="52" t="n"/>
-      <c r="D45" s="53" t="inlineStr">
+      <c r="A45" s="58" t="n"/>
+      <c r="B45" s="58" t="n"/>
+      <c r="C45" s="58" t="n"/>
+      <c r="D45" s="60" t="inlineStr">
         <is>
           <t>Data: 15/04/2026</t>
         </is>
       </c>
-      <c r="E45" s="52" t="n"/>
-      <c r="F45" s="52" t="n"/>
-      <c r="G45" s="52" t="n"/>
-      <c r="H45" s="52" t="n"/>
+      <c r="E45" s="58" t="n"/>
+      <c r="F45" s="58" t="n"/>
+      <c r="G45" s="58" t="n"/>
+      <c r="H45" s="58" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="19" t="inlineStr">

</xml_diff>

<commit_message>
ajuste instrumento de pressão diferencial (com saida elétrica) por delimitação de range <= 200
</commit_message>
<xml_diff>
--- a/TemplateAC_ORIGEM.xlsx
+++ b/TemplateAC_ORIGEM.xlsx
@@ -372,7 +372,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -516,6 +516,15 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -1006,25 +1015,25 @@
     <row r="6" ht="34.5" customHeight="1" s="20">
       <c r="A6" s="32" t="inlineStr">
         <is>
-          <t>UT-SG-122101-01</t>
+          <t>FT-SG-122101-001A</t>
         </is>
       </c>
       <c r="B6" s="13" t="n"/>
       <c r="C6" s="32" t="inlineStr">
         <is>
-          <t>TESTE</t>
+          <t>teste</t>
         </is>
       </c>
       <c r="D6" s="12" t="n"/>
       <c r="E6" s="13" t="n"/>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>SAP: TESTE</t>
+          <t>SAP: teste</t>
         </is>
       </c>
       <c r="G6" s="32" t="inlineStr">
         <is>
-          <t>CE: TESTE</t>
+          <t>CE: teste</t>
         </is>
       </c>
       <c r="H6" s="13" t="n"/>
@@ -1112,14 +1121,14 @@
     <row r="13">
       <c r="A13" s="32" t="inlineStr">
         <is>
-          <t>26-ODS-0638-PRE-444</t>
+          <t>26-ODS-0638-PRE-443</t>
         </is>
       </c>
       <c r="B13" s="12" t="n"/>
       <c r="C13" s="13" t="n"/>
       <c r="D13" s="16" t="inlineStr">
         <is>
-          <t>09/04/2026</t>
+          <t>07/04/2026</t>
         </is>
       </c>
       <c r="E13" s="17" t="n"/>
@@ -1734,18 +1743,18 @@
       <c r="H43" s="31" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="58" t="n"/>
-      <c r="B45" s="58" t="n"/>
-      <c r="C45" s="58" t="n"/>
-      <c r="D45" s="60" t="inlineStr">
-        <is>
-          <t>Data: 15/04/2026</t>
-        </is>
-      </c>
-      <c r="E45" s="58" t="n"/>
-      <c r="F45" s="58" t="n"/>
-      <c r="G45" s="58" t="n"/>
-      <c r="H45" s="58" t="n"/>
+      <c r="A45" s="62" t="n"/>
+      <c r="B45" s="62" t="n"/>
+      <c r="C45" s="62" t="n"/>
+      <c r="D45" s="63" t="inlineStr">
+        <is>
+          <t>Data: 14/04/2026</t>
+        </is>
+      </c>
+      <c r="E45" s="62" t="n"/>
+      <c r="F45" s="62" t="n"/>
+      <c r="G45" s="62" t="n"/>
+      <c r="H45" s="62" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="19" t="inlineStr">

</xml_diff>

<commit_message>
ajuste de preenchimento dos equipamentos que possuem ajuste na calibração - AC ORIGEM
</commit_message>
<xml_diff>
--- a/TemplateAC_ORIGEM.xlsx
+++ b/TemplateAC_ORIGEM.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="380" yWindow="380" windowWidth="14400" windowHeight="7270" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template Formulário" sheetId="1" state="visible" r:id="rId1"/>
@@ -372,12 +372,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -385,9 +382,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -396,38 +390,48 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -486,36 +490,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -936,59 +910,59 @@
   <dimension ref="A1:O49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
-    <col width="15" customWidth="1" style="20" min="1" max="4"/>
-    <col width="11.7265625" customWidth="1" style="20" min="5" max="5"/>
-    <col width="12.453125" customWidth="1" style="20" min="6" max="6"/>
-    <col width="4.90625" bestFit="1" customWidth="1" style="20" min="7" max="7"/>
-    <col width="15" customWidth="1" style="20" min="8" max="8"/>
+    <col width="15" customWidth="1" style="23" min="1" max="4"/>
+    <col width="11.7265625" customWidth="1" style="23" min="5" max="5"/>
+    <col width="12.453125" customWidth="1" style="23" min="6" max="6"/>
+    <col width="4.90625" bestFit="1" customWidth="1" style="23" min="7" max="7"/>
+    <col width="15" customWidth="1" style="23" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20" customHeight="1" s="20">
-      <c r="A1" s="27" t="n"/>
-      <c r="B1" s="28" t="n"/>
-      <c r="C1" s="44" t="inlineStr">
+    <row r="1" ht="20" customHeight="1" s="23">
+      <c r="A1" s="29" t="n"/>
+      <c r="B1" s="30" t="n"/>
+      <c r="C1" s="46" t="inlineStr">
         <is>
           <t>REGISTRO DE ANÁLISE CRÍTICA DE CERTIFICADO DE CALIBRAÇÃO DE SECUNDÁRIOS</t>
         </is>
       </c>
-      <c r="D1" s="34" t="n"/>
-      <c r="E1" s="34" t="n"/>
-      <c r="F1" s="28" t="n"/>
-      <c r="G1" s="43" t="inlineStr">
+      <c r="D1" s="36" t="n"/>
+      <c r="E1" s="36" t="n"/>
+      <c r="F1" s="30" t="n"/>
+      <c r="G1" s="45" t="inlineStr">
         <is>
           <t>FO-COR-GER-CPROD-030</t>
         </is>
       </c>
-      <c r="H1" s="28" t="n"/>
-    </row>
-    <row r="2" ht="20" customHeight="1" s="20">
-      <c r="A2" s="29" t="n"/>
-      <c r="B2" s="23" t="n"/>
-      <c r="C2" s="29" t="n"/>
-      <c r="F2" s="23" t="n"/>
-      <c r="G2" s="22" t="inlineStr">
+      <c r="H1" s="30" t="n"/>
+    </row>
+    <row r="2" ht="20" customHeight="1" s="23">
+      <c r="A2" s="31" t="n"/>
+      <c r="B2" s="25" t="n"/>
+      <c r="C2" s="31" t="n"/>
+      <c r="F2" s="25" t="n"/>
+      <c r="G2" s="24" t="inlineStr">
         <is>
           <t>Revisão: 0</t>
         </is>
       </c>
-      <c r="H2" s="23" t="n"/>
-    </row>
-    <row r="3" ht="20" customHeight="1" s="20">
-      <c r="A3" s="30" t="n"/>
-      <c r="B3" s="31" t="n"/>
-      <c r="C3" s="30" t="n"/>
-      <c r="D3" s="35" t="n"/>
-      <c r="E3" s="35" t="n"/>
-      <c r="F3" s="31" t="n"/>
-      <c r="G3" s="41" t="inlineStr">
+      <c r="H2" s="25" t="n"/>
+    </row>
+    <row r="3" ht="20" customHeight="1" s="23">
+      <c r="A3" s="32" t="n"/>
+      <c r="B3" s="33" t="n"/>
+      <c r="C3" s="32" t="n"/>
+      <c r="D3" s="37" t="n"/>
+      <c r="E3" s="37" t="n"/>
+      <c r="F3" s="33" t="n"/>
+      <c r="G3" s="43" t="inlineStr">
         <is>
           <t>Página: 1/1</t>
         </is>
       </c>
-      <c r="H3" s="31" t="n"/>
+      <c r="H3" s="33" t="n"/>
     </row>
     <row r="4">
-      <c r="G4" s="2" t="n"/>
+      <c r="G4" s="1" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="21" t="inlineStr">
@@ -996,105 +970,105 @@
           <t>TAG</t>
         </is>
       </c>
-      <c r="B5" s="13" t="n"/>
+      <c r="B5" s="15" t="n"/>
       <c r="C5" s="21" t="inlineStr">
         <is>
           <t>Localização</t>
         </is>
       </c>
-      <c r="D5" s="12" t="n"/>
-      <c r="E5" s="13" t="n"/>
+      <c r="D5" s="14" t="n"/>
+      <c r="E5" s="15" t="n"/>
       <c r="F5" s="21" t="inlineStr">
         <is>
           <t>Identificação</t>
         </is>
       </c>
-      <c r="G5" s="12" t="n"/>
-      <c r="H5" s="13" t="n"/>
-    </row>
-    <row r="6" ht="34.5" customHeight="1" s="20">
-      <c r="A6" s="32" t="inlineStr">
-        <is>
-          <t>FT-SG-122101-001A</t>
-        </is>
-      </c>
-      <c r="B6" s="13" t="n"/>
-      <c r="C6" s="32" t="inlineStr">
-        <is>
-          <t>teste</t>
-        </is>
-      </c>
-      <c r="D6" s="12" t="n"/>
-      <c r="E6" s="13" t="n"/>
-      <c r="F6" s="8" t="inlineStr">
-        <is>
-          <t>SAP: teste</t>
-        </is>
-      </c>
-      <c r="G6" s="32" t="inlineStr">
-        <is>
-          <t>CE: teste</t>
-        </is>
-      </c>
-      <c r="H6" s="13" t="n"/>
-    </row>
-    <row r="7" ht="14.5" customHeight="1" s="20">
-      <c r="A7" s="2" t="n"/>
-      <c r="B7" s="2" t="n"/>
-      <c r="C7" s="2" t="n"/>
-      <c r="D7" s="2" t="n"/>
-      <c r="E7" s="2" t="n"/>
-      <c r="F7" s="3" t="n"/>
-      <c r="G7" s="3" t="n"/>
-      <c r="H7" s="3" t="n"/>
-    </row>
-    <row r="8" ht="14.5" customHeight="1" s="20">
-      <c r="A8" s="42" t="inlineStr">
+      <c r="G5" s="14" t="n"/>
+      <c r="H5" s="15" t="n"/>
+    </row>
+    <row r="6" ht="34.5" customHeight="1" s="23">
+      <c r="A6" s="34" t="inlineStr">
+        <is>
+          <t>FT-C-624005-02</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="n"/>
+      <c r="C6" s="34" t="inlineStr">
+        <is>
+          <t>loc</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="n"/>
+      <c r="E6" s="15" t="n"/>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>SAP: sap</t>
+        </is>
+      </c>
+      <c r="G6" s="34" t="inlineStr">
+        <is>
+          <t>CE: nac</t>
+        </is>
+      </c>
+      <c r="H6" s="15" t="n"/>
+    </row>
+    <row r="7" ht="14.5" customHeight="1" s="23">
+      <c r="A7" s="1" t="n"/>
+      <c r="B7" s="1" t="n"/>
+      <c r="C7" s="1" t="n"/>
+      <c r="D7" s="1" t="n"/>
+      <c r="E7" s="1" t="n"/>
+      <c r="F7" s="2" t="n"/>
+      <c r="G7" s="2" t="n"/>
+      <c r="H7" s="2" t="n"/>
+    </row>
+    <row r="8" ht="14.5" customHeight="1" s="23">
+      <c r="A8" s="44" t="inlineStr">
         <is>
           <t>OUTRAS INFORMAÇÕES (Descrição):</t>
         </is>
       </c>
-      <c r="B8" s="28" t="n"/>
-      <c r="C8" s="37" t="inlineStr">
+      <c r="B8" s="30" t="n"/>
+      <c r="C8" s="39" t="inlineStr">
         <is>
           <t>[ ] Transmissor de pressão estática (PT)</t>
         </is>
       </c>
-      <c r="D8" s="34" t="n"/>
-      <c r="E8" s="28" t="n"/>
-      <c r="F8" s="32" t="inlineStr">
+      <c r="D8" s="36" t="n"/>
+      <c r="E8" s="30" t="n"/>
+      <c r="F8" s="34" t="inlineStr">
         <is>
           <t>[ ] Termorresistência (TE)</t>
         </is>
       </c>
-      <c r="G8" s="34" t="n"/>
-      <c r="H8" s="28" t="n"/>
+      <c r="G8" s="36" t="n"/>
+      <c r="H8" s="30" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="29" t="n"/>
-      <c r="B9" s="23" t="n"/>
-      <c r="C9" s="25" t="inlineStr">
+      <c r="A9" s="31" t="n"/>
+      <c r="B9" s="25" t="n"/>
+      <c r="C9" s="27" t="inlineStr">
         <is>
           <t>[ ✔ ] Transmissor de pressão diferencial (PDT)</t>
         </is>
       </c>
-      <c r="E9" s="23" t="n"/>
-      <c r="F9" s="29" t="n"/>
-      <c r="H9" s="23" t="n"/>
+      <c r="E9" s="25" t="n"/>
+      <c r="F9" s="31" t="n"/>
+      <c r="H9" s="25" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="30" t="n"/>
-      <c r="B10" s="31" t="n"/>
-      <c r="C10" s="45" t="inlineStr">
+      <c r="A10" s="32" t="n"/>
+      <c r="B10" s="33" t="n"/>
+      <c r="C10" s="47" t="inlineStr">
         <is>
           <t>[ ] Transmissor de temperatura (TT)</t>
         </is>
       </c>
-      <c r="D10" s="35" t="n"/>
-      <c r="E10" s="31" t="n"/>
-      <c r="F10" s="30" t="n"/>
-      <c r="G10" s="35" t="n"/>
-      <c r="H10" s="31" t="n"/>
+      <c r="D10" s="37" t="n"/>
+      <c r="E10" s="33" t="n"/>
+      <c r="F10" s="32" t="n"/>
+      <c r="G10" s="37" t="n"/>
+      <c r="H10" s="33" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="21" t="inlineStr">
@@ -1102,38 +1076,38 @@
           <t>Nº do Certificado</t>
         </is>
       </c>
-      <c r="B12" s="12" t="n"/>
-      <c r="C12" s="13" t="n"/>
-      <c r="D12" s="38" t="inlineStr">
+      <c r="B12" s="14" t="n"/>
+      <c r="C12" s="15" t="n"/>
+      <c r="D12" s="40" t="inlineStr">
         <is>
           <t>Data da Calibração</t>
         </is>
       </c>
-      <c r="E12" s="39" t="n"/>
-      <c r="F12" s="15" t="n"/>
-      <c r="G12" s="14" t="inlineStr">
+      <c r="E12" s="41" t="n"/>
+      <c r="F12" s="20" t="n"/>
+      <c r="G12" s="19" t="inlineStr">
         <is>
           <t>Empresa Certificadora</t>
         </is>
       </c>
-      <c r="H12" s="15" t="n"/>
+      <c r="H12" s="20" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="32" t="inlineStr">
-        <is>
-          <t>26-ODS-0638-PRE-443</t>
-        </is>
-      </c>
-      <c r="B13" s="12" t="n"/>
-      <c r="C13" s="13" t="n"/>
+      <c r="A13" s="34" t="inlineStr">
+        <is>
+          <t>26-ODS-0638-PRE-040</t>
+        </is>
+      </c>
+      <c r="B13" s="14" t="n"/>
+      <c r="C13" s="15" t="n"/>
       <c r="D13" s="16" t="inlineStr">
         <is>
-          <t>07/04/2026</t>
+          <t>09/04/2026</t>
         </is>
       </c>
       <c r="E13" s="17" t="n"/>
       <c r="F13" s="18" t="n"/>
-      <c r="G13" s="40" t="inlineStr">
+      <c r="G13" s="42" t="inlineStr">
         <is>
           <t>ODS Lab</t>
         </is>
@@ -1141,623 +1115,623 @@
       <c r="H13" s="18" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="n"/>
-      <c r="B14" s="2" t="n"/>
-      <c r="C14" s="2" t="n"/>
-      <c r="D14" s="2" t="n"/>
-      <c r="E14" s="2" t="n"/>
-      <c r="F14" s="2" t="n"/>
-      <c r="G14" s="2" t="n"/>
-      <c r="H14" s="2" t="n"/>
+      <c r="A14" s="1" t="n"/>
+      <c r="B14" s="1" t="n"/>
+      <c r="C14" s="1" t="n"/>
+      <c r="D14" s="1" t="n"/>
+      <c r="E14" s="1" t="n"/>
+      <c r="F14" s="1" t="n"/>
+      <c r="G14" s="1" t="n"/>
+      <c r="H14" s="1" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="24" t="inlineStr">
+      <c r="A15" s="22" t="inlineStr">
         <is>
           <t>1 - ANÁLISE DO CERTIFICADO DE CALIBRAÇÃO</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="25" customHeight="1" s="20">
-      <c r="A16" s="36" t="inlineStr">
+    <row r="16" ht="25" customHeight="1" s="23">
+      <c r="A16" s="38" t="inlineStr">
         <is>
           <t>DESCRIÇÃO DOS ITENS A SEREM VERIFICADOS</t>
         </is>
       </c>
-      <c r="B16" s="12" t="n"/>
-      <c r="C16" s="12" t="n"/>
-      <c r="D16" s="12" t="n"/>
-      <c r="E16" s="13" t="n"/>
-      <c r="F16" s="36" t="inlineStr">
+      <c r="B16" s="14" t="n"/>
+      <c r="C16" s="14" t="n"/>
+      <c r="D16" s="14" t="n"/>
+      <c r="E16" s="15" t="n"/>
+      <c r="F16" s="38" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
       </c>
-      <c r="G16" s="36" t="inlineStr">
+      <c r="G16" s="38" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
-      <c r="H16" s="36" t="inlineStr">
+      <c r="H16" s="38" t="inlineStr">
         <is>
           <t>NÃO APLICÁVEL</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="16.5" customHeight="1" s="20">
-      <c r="A17" s="11" t="inlineStr">
+    <row r="17" ht="16.5" customHeight="1" s="23">
+      <c r="A17" s="13" t="inlineStr">
         <is>
           <t>a) Identificação unívoca (Número do Certificado de Calibração).</t>
         </is>
       </c>
-      <c r="B17" s="12" t="n"/>
-      <c r="C17" s="12" t="n"/>
-      <c r="D17" s="12" t="n"/>
-      <c r="E17" s="13" t="n"/>
-      <c r="F17" s="7" t="inlineStr">
+      <c r="B17" s="14" t="n"/>
+      <c r="C17" s="14" t="n"/>
+      <c r="D17" s="14" t="n"/>
+      <c r="E17" s="15" t="n"/>
+      <c r="F17" s="5" t="inlineStr">
         <is>
           <t>◉</t>
         </is>
       </c>
-      <c r="G17" s="7" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="H17" s="7" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="16.5" customHeight="1" s="20">
-      <c r="A18" s="11" t="inlineStr">
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="16.5" customHeight="1" s="23">
+      <c r="A18" s="13" t="inlineStr">
         <is>
           <t>b) Nome e endereço do Laboratório/Empresa.</t>
         </is>
       </c>
-      <c r="B18" s="12" t="n"/>
-      <c r="C18" s="12" t="n"/>
-      <c r="D18" s="12" t="n"/>
-      <c r="E18" s="13" t="n"/>
-      <c r="F18" s="7" t="inlineStr">
+      <c r="B18" s="14" t="n"/>
+      <c r="C18" s="14" t="n"/>
+      <c r="D18" s="14" t="n"/>
+      <c r="E18" s="15" t="n"/>
+      <c r="F18" s="5" t="inlineStr">
         <is>
           <t>◉</t>
         </is>
       </c>
-      <c r="G18" s="7" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="H18" s="7" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="31" customHeight="1" s="20">
-      <c r="A19" s="11" t="inlineStr">
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="31" customHeight="1" s="23">
+      <c r="A19" s="13" t="inlineStr">
         <is>
           <t>c) Logotipo da RBC (para instrumento associado a sistemas de medição fiscal, apropriação, custódia, flare)</t>
         </is>
       </c>
-      <c r="B19" s="12" t="n"/>
-      <c r="C19" s="12" t="n"/>
-      <c r="D19" s="12" t="n"/>
-      <c r="E19" s="13" t="n"/>
-      <c r="F19" s="7" t="inlineStr">
+      <c r="B19" s="14" t="n"/>
+      <c r="C19" s="14" t="n"/>
+      <c r="D19" s="14" t="n"/>
+      <c r="E19" s="15" t="n"/>
+      <c r="F19" s="5" t="inlineStr">
         <is>
           <t>◉</t>
         </is>
       </c>
-      <c r="G19" s="7" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="H19" s="7" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="16.5" customHeight="1" s="20">
-      <c r="A20" s="11" t="inlineStr">
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="16.5" customHeight="1" s="23">
+      <c r="A20" s="13" t="inlineStr">
         <is>
           <t>d) Nome e endereço do cliente.</t>
         </is>
       </c>
-      <c r="B20" s="12" t="n"/>
-      <c r="C20" s="12" t="n"/>
-      <c r="D20" s="12" t="n"/>
-      <c r="E20" s="13" t="n"/>
-      <c r="F20" s="7" t="inlineStr">
+      <c r="B20" s="14" t="n"/>
+      <c r="C20" s="14" t="n"/>
+      <c r="D20" s="14" t="n"/>
+      <c r="E20" s="15" t="n"/>
+      <c r="F20" s="5" t="inlineStr">
         <is>
           <t>◉</t>
         </is>
       </c>
-      <c r="G20" s="7" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="H20" s="7" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="16.5" customHeight="1" s="20">
-      <c r="A21" s="11" t="inlineStr">
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="16.5" customHeight="1" s="23">
+      <c r="A21" s="13" t="inlineStr">
         <is>
           <t>e) Número de páginas e total de páginas.</t>
         </is>
       </c>
-      <c r="B21" s="12" t="n"/>
-      <c r="C21" s="12" t="n"/>
-      <c r="D21" s="12" t="n"/>
-      <c r="E21" s="13" t="n"/>
-      <c r="F21" s="7" t="inlineStr">
+      <c r="B21" s="14" t="n"/>
+      <c r="C21" s="14" t="n"/>
+      <c r="D21" s="14" t="n"/>
+      <c r="E21" s="15" t="n"/>
+      <c r="F21" s="5" t="inlineStr">
         <is>
           <t>◉</t>
         </is>
       </c>
-      <c r="G21" s="7" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="H21" s="7" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="16.5" customHeight="1" s="20">
-      <c r="A22" s="11" t="inlineStr">
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="16.5" customHeight="1" s="23">
+      <c r="A22" s="13" t="inlineStr">
         <is>
           <t>f) Identificação do método/procedimento utilizado.</t>
         </is>
       </c>
-      <c r="B22" s="12" t="n"/>
-      <c r="C22" s="12" t="n"/>
-      <c r="D22" s="12" t="n"/>
-      <c r="E22" s="13" t="n"/>
-      <c r="F22" s="7" t="inlineStr">
+      <c r="B22" s="14" t="n"/>
+      <c r="C22" s="14" t="n"/>
+      <c r="D22" s="14" t="n"/>
+      <c r="E22" s="15" t="n"/>
+      <c r="F22" s="5" t="inlineStr">
         <is>
           <t>◉</t>
         </is>
       </c>
-      <c r="G22" s="7" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="H22" s="7" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="16.5" customHeight="1" s="20">
-      <c r="A23" s="11" t="inlineStr">
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="16.5" customHeight="1" s="23">
+      <c r="A23" s="13" t="inlineStr">
         <is>
           <t>g) Registro das condições ambientais.</t>
         </is>
       </c>
-      <c r="B23" s="12" t="n"/>
-      <c r="C23" s="12" t="n"/>
-      <c r="D23" s="12" t="n"/>
-      <c r="E23" s="13" t="n"/>
-      <c r="F23" s="7" t="inlineStr">
+      <c r="B23" s="14" t="n"/>
+      <c r="C23" s="14" t="n"/>
+      <c r="D23" s="14" t="n"/>
+      <c r="E23" s="15" t="n"/>
+      <c r="F23" s="5" t="inlineStr">
         <is>
           <t>◉</t>
         </is>
       </c>
-      <c r="G23" s="7" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="H23" s="7" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="31" customHeight="1" s="20">
-      <c r="A24" s="11" t="inlineStr">
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="31" customHeight="1" s="23">
+      <c r="A24" s="13" t="inlineStr">
         <is>
           <t>h) Descrição e identificação do item de calibração (ex.: nome, fabricante, tipo, modelo, número de série, outra identificação estabelecida pelo cliente).</t>
         </is>
       </c>
-      <c r="B24" s="12" t="n"/>
-      <c r="C24" s="12" t="n"/>
-      <c r="D24" s="12" t="n"/>
-      <c r="E24" s="13" t="n"/>
-      <c r="F24" s="7" t="inlineStr">
+      <c r="B24" s="14" t="n"/>
+      <c r="C24" s="14" t="n"/>
+      <c r="D24" s="14" t="n"/>
+      <c r="E24" s="15" t="n"/>
+      <c r="F24" s="5" t="inlineStr">
         <is>
           <t>◉</t>
         </is>
       </c>
-      <c r="G24" s="7" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="H24" s="7" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="16.5" customHeight="1" s="20">
-      <c r="A25" s="11" t="inlineStr">
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="16.5" customHeight="1" s="23">
+      <c r="A25" s="13" t="inlineStr">
         <is>
           <t>i) A data do recebimento do(s) item(s) de calibração, se necessário.</t>
         </is>
       </c>
-      <c r="B25" s="12" t="n"/>
-      <c r="C25" s="12" t="n"/>
-      <c r="D25" s="12" t="n"/>
-      <c r="E25" s="13" t="n"/>
-      <c r="F25" s="7" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="G25" s="7" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="H25" s="7" t="inlineStr">
+      <c r="B25" s="14" t="n"/>
+      <c r="C25" s="14" t="n"/>
+      <c r="D25" s="14" t="n"/>
+      <c r="E25" s="15" t="n"/>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="inlineStr">
         <is>
           <t>◉</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="16.5" customHeight="1" s="20">
-      <c r="A26" s="11" t="inlineStr">
+    <row r="26" ht="16.5" customHeight="1" s="23">
+      <c r="A26" s="13" t="inlineStr">
         <is>
           <t>j) A data da realização da calibração.</t>
         </is>
       </c>
-      <c r="B26" s="12" t="n"/>
-      <c r="C26" s="12" t="n"/>
-      <c r="D26" s="12" t="n"/>
-      <c r="E26" s="13" t="n"/>
-      <c r="F26" s="7" t="inlineStr">
+      <c r="B26" s="14" t="n"/>
+      <c r="C26" s="14" t="n"/>
+      <c r="D26" s="14" t="n"/>
+      <c r="E26" s="15" t="n"/>
+      <c r="F26" s="5" t="inlineStr">
         <is>
           <t>◉</t>
         </is>
       </c>
-      <c r="G26" s="7" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="H26" s="7" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="31" customHeight="1" s="20">
-      <c r="A27" s="11" t="inlineStr">
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="31" customHeight="1" s="23">
+      <c r="A27" s="13" t="inlineStr">
         <is>
           <t>k) Os resultados da calibração estão com as unidades de medida no SI, onde apropriado.</t>
         </is>
       </c>
-      <c r="B27" s="12" t="n"/>
-      <c r="C27" s="12" t="n"/>
-      <c r="D27" s="12" t="n"/>
-      <c r="E27" s="13" t="n"/>
-      <c r="F27" s="7" t="inlineStr">
+      <c r="B27" s="14" t="n"/>
+      <c r="C27" s="14" t="n"/>
+      <c r="D27" s="14" t="n"/>
+      <c r="E27" s="15" t="n"/>
+      <c r="F27" s="5" t="inlineStr">
         <is>
           <t>◉</t>
         </is>
       </c>
-      <c r="G27" s="7" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="H27" s="7" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="16.5" customHeight="1" s="20">
-      <c r="A28" s="11" t="inlineStr">
+      <c r="G27" s="5" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H27" s="5" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="16.5" customHeight="1" s="23">
+      <c r="A28" s="13" t="inlineStr">
         <is>
           <t>l) Evidências de que as medições são rastreáveis (Informações dos padrões utilizados).</t>
         </is>
       </c>
-      <c r="B28" s="12" t="n"/>
-      <c r="C28" s="12" t="n"/>
-      <c r="D28" s="12" t="n"/>
-      <c r="E28" s="13" t="n"/>
-      <c r="F28" s="7" t="inlineStr">
+      <c r="B28" s="14" t="n"/>
+      <c r="C28" s="14" t="n"/>
+      <c r="D28" s="14" t="n"/>
+      <c r="E28" s="15" t="n"/>
+      <c r="F28" s="5" t="inlineStr">
         <is>
           <t>◉</t>
         </is>
       </c>
-      <c r="G28" s="7" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="H28" s="7" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="31" customHeight="1" s="20">
-      <c r="A29" s="11" t="inlineStr">
+      <c r="G28" s="5" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H28" s="5" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="31" customHeight="1" s="23">
+      <c r="A29" s="13" t="inlineStr">
         <is>
           <t>m) Nome(s), função (ões) e assinatura (s) ou identificações equivalentes das pessoas autorizadas para emissão do certificado.</t>
         </is>
       </c>
-      <c r="B29" s="12" t="n"/>
-      <c r="C29" s="12" t="n"/>
-      <c r="D29" s="12" t="n"/>
-      <c r="E29" s="13" t="n"/>
-      <c r="F29" s="7" t="inlineStr">
+      <c r="B29" s="14" t="n"/>
+      <c r="C29" s="14" t="n"/>
+      <c r="D29" s="14" t="n"/>
+      <c r="E29" s="15" t="n"/>
+      <c r="F29" s="5" t="inlineStr">
         <is>
           <t>◉</t>
         </is>
       </c>
-      <c r="G29" s="7" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="H29" s="7" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="31" customHeight="1" s="20">
-      <c r="A30" s="11" t="inlineStr">
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H29" s="5" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="31" customHeight="1" s="23">
+      <c r="A30" s="13" t="inlineStr">
         <is>
           <t>n) Declaração de que os resultados e incertezas se referem somente aos itens calibrados / inspecionados.</t>
         </is>
       </c>
-      <c r="B30" s="12" t="n"/>
-      <c r="C30" s="12" t="n"/>
-      <c r="D30" s="12" t="n"/>
-      <c r="E30" s="13" t="n"/>
-      <c r="F30" s="7" t="inlineStr">
+      <c r="B30" s="14" t="n"/>
+      <c r="C30" s="14" t="n"/>
+      <c r="D30" s="14" t="n"/>
+      <c r="E30" s="15" t="n"/>
+      <c r="F30" s="5" t="inlineStr">
         <is>
           <t>◉</t>
         </is>
       </c>
-      <c r="G30" s="7" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="H30" s="7" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="16.5" customHeight="1" s="20">
-      <c r="A31" s="11" t="inlineStr">
+      <c r="G30" s="5" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H30" s="5" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="16.5" customHeight="1" s="23">
+      <c r="A31" s="13" t="inlineStr">
         <is>
           <t>o) Nível de confiança e fator de abrangência.</t>
         </is>
       </c>
-      <c r="B31" s="12" t="n"/>
-      <c r="C31" s="12" t="n"/>
-      <c r="D31" s="12" t="n"/>
-      <c r="E31" s="13" t="n"/>
-      <c r="F31" s="7" t="inlineStr">
+      <c r="B31" s="14" t="n"/>
+      <c r="C31" s="14" t="n"/>
+      <c r="D31" s="14" t="n"/>
+      <c r="E31" s="15" t="n"/>
+      <c r="F31" s="5" t="inlineStr">
         <is>
           <t>◉</t>
         </is>
       </c>
-      <c r="G31" s="7" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="H31" s="7" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="16.5" customHeight="1" s="20">
-      <c r="A32" s="11" t="inlineStr">
+      <c r="G31" s="5" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H31" s="5" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="16.5" customHeight="1" s="23">
+      <c r="A32" s="13" t="inlineStr">
         <is>
           <t>p) Foi feita calibração de acordo com a faixa solicitada?</t>
         </is>
       </c>
-      <c r="B32" s="12" t="n"/>
-      <c r="C32" s="12" t="n"/>
-      <c r="D32" s="12" t="n"/>
-      <c r="E32" s="13" t="n"/>
-      <c r="F32" s="7" t="inlineStr">
+      <c r="B32" s="14" t="n"/>
+      <c r="C32" s="14" t="n"/>
+      <c r="D32" s="14" t="n"/>
+      <c r="E32" s="15" t="n"/>
+      <c r="F32" s="5" t="inlineStr">
         <is>
           <t>◉</t>
         </is>
       </c>
-      <c r="G32" s="7" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="H32" s="7" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="31" customHeight="1" s="20">
-      <c r="A33" s="11" t="inlineStr">
+      <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H32" s="5" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="31" customHeight="1" s="23">
+      <c r="A33" s="13" t="inlineStr">
         <is>
           <t>q) Os erros máximos de medição (Erro sistemático remanescente + incerteza) são inferiores ao erro máximo admissível para o equipamento em questão?</t>
         </is>
       </c>
-      <c r="B33" s="12" t="n"/>
-      <c r="C33" s="12" t="n"/>
-      <c r="D33" s="12" t="n"/>
-      <c r="E33" s="13" t="n"/>
-      <c r="F33" s="7" t="inlineStr">
+      <c r="B33" s="14" t="n"/>
+      <c r="C33" s="14" t="n"/>
+      <c r="D33" s="14" t="n"/>
+      <c r="E33" s="15" t="n"/>
+      <c r="F33" s="5" t="inlineStr">
         <is>
           <t>◉</t>
         </is>
       </c>
-      <c r="G33" s="7" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="H33" s="7" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="31" customHeight="1" s="20">
-      <c r="A34" s="11" t="inlineStr">
+      <c r="G33" s="5" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H33" s="5" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="31" customHeight="1" s="23">
+      <c r="A34" s="13" t="inlineStr">
         <is>
           <t>r) O instrumento está aprovado para o uso no ponto de medição a que se destina de acordo com os critérios de aceitação informados pelo cliente?</t>
         </is>
       </c>
-      <c r="B34" s="12" t="n"/>
-      <c r="C34" s="12" t="n"/>
-      <c r="D34" s="12" t="n"/>
-      <c r="E34" s="13" t="n"/>
-      <c r="F34" s="7" t="inlineStr">
+      <c r="B34" s="14" t="n"/>
+      <c r="C34" s="14" t="n"/>
+      <c r="D34" s="14" t="n"/>
+      <c r="E34" s="15" t="n"/>
+      <c r="F34" s="5" t="inlineStr">
         <is>
           <t>◉</t>
         </is>
       </c>
-      <c r="G34" s="7" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="H34" s="7" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="31" customHeight="1" s="20">
-      <c r="A35" s="11" t="inlineStr">
+      <c r="G34" s="5" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H34" s="5" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="31" customHeight="1" s="23">
+      <c r="A35" s="13" t="inlineStr">
         <is>
           <t>s) No caso de ajuste no equipamento, estão informados os resultados das calibrações como encontrados (as found) e como deixados (as left)?</t>
         </is>
       </c>
-      <c r="B35" s="12" t="n"/>
-      <c r="C35" s="12" t="n"/>
-      <c r="D35" s="12" t="n"/>
-      <c r="E35" s="13" t="n"/>
-      <c r="F35" s="59" t="inlineStr">
+      <c r="B35" s="14" t="n"/>
+      <c r="C35" s="14" t="n"/>
+      <c r="D35" s="14" t="n"/>
+      <c r="E35" s="15" t="n"/>
+      <c r="F35" s="10" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="G35" s="10" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H35" s="10" t="inlineStr">
         <is>
           <t>◉</t>
         </is>
       </c>
-      <c r="G35" s="10" t="inlineStr">
-        <is>
-          <t>●</t>
-        </is>
-      </c>
-      <c r="H35" s="59" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
     </row>
     <row r="36">
-      <c r="A36" s="4" t="n"/>
-      <c r="F36" s="2" t="n"/>
-      <c r="G36" s="2" t="n"/>
-      <c r="H36" s="2" t="n"/>
+      <c r="A36" s="3" t="n"/>
+      <c r="F36" s="1" t="n"/>
+      <c r="G36" s="1" t="n"/>
+      <c r="H36" s="1" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="24" t="inlineStr">
+      <c r="A37" s="22" t="inlineStr">
         <is>
           <t>1.1 Conclusão da análise crítica do certificado de calibração:</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="26" t="inlineStr">
+      <c r="A38" s="28" t="inlineStr">
         <is>
           <t xml:space="preserve">O certificado está conforme e atende ao procedimento?  </t>
         </is>
       </c>
     </row>
-    <row r="39" ht="16.5" customHeight="1" s="20">
-      <c r="A39" s="19" t="inlineStr">
+    <row r="39" ht="16.5" customHeight="1" s="23">
+      <c r="A39" s="26" t="inlineStr">
         <is>
           <t>◉ Sim  ○ Não</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="19" t="n"/>
-      <c r="B40" s="19" t="n"/>
-      <c r="C40" s="19" t="n"/>
-      <c r="D40" s="19" t="n"/>
-      <c r="E40" s="19" t="n"/>
-      <c r="F40" s="19" t="n"/>
-      <c r="G40" s="19" t="n"/>
-      <c r="H40" s="19" t="n"/>
-      <c r="O40" s="6" t="n"/>
+      <c r="A40" s="26" t="n"/>
+      <c r="B40" s="26" t="n"/>
+      <c r="C40" s="26" t="n"/>
+      <c r="D40" s="26" t="n"/>
+      <c r="E40" s="26" t="n"/>
+      <c r="F40" s="26" t="n"/>
+      <c r="G40" s="26" t="n"/>
+      <c r="H40" s="26" t="n"/>
+      <c r="O40" s="4" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="24" t="inlineStr">
+      <c r="A41" s="22" t="inlineStr">
         <is>
           <t>OBSERVAÇÕES:</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="33" t="inlineStr"/>
-      <c r="B42" s="34" t="n"/>
-      <c r="C42" s="34" t="n"/>
-      <c r="D42" s="34" t="n"/>
-      <c r="E42" s="34" t="n"/>
-      <c r="F42" s="34" t="n"/>
-      <c r="G42" s="34" t="n"/>
-      <c r="H42" s="28" t="n"/>
+      <c r="A42" s="35" t="inlineStr"/>
+      <c r="B42" s="36" t="n"/>
+      <c r="C42" s="36" t="n"/>
+      <c r="D42" s="36" t="n"/>
+      <c r="E42" s="36" t="n"/>
+      <c r="F42" s="36" t="n"/>
+      <c r="G42" s="36" t="n"/>
+      <c r="H42" s="30" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="30" t="n"/>
-      <c r="B43" s="35" t="n"/>
-      <c r="C43" s="35" t="n"/>
-      <c r="D43" s="35" t="n"/>
-      <c r="E43" s="35" t="n"/>
-      <c r="F43" s="35" t="n"/>
-      <c r="G43" s="35" t="n"/>
-      <c r="H43" s="31" t="n"/>
+      <c r="A43" s="32" t="n"/>
+      <c r="B43" s="37" t="n"/>
+      <c r="C43" s="37" t="n"/>
+      <c r="D43" s="37" t="n"/>
+      <c r="E43" s="37" t="n"/>
+      <c r="F43" s="37" t="n"/>
+      <c r="G43" s="37" t="n"/>
+      <c r="H43" s="33" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="62" t="n"/>
-      <c r="B45" s="62" t="n"/>
-      <c r="C45" s="62" t="n"/>
-      <c r="D45" s="63" t="inlineStr">
-        <is>
-          <t>Data: 14/04/2026</t>
-        </is>
-      </c>
-      <c r="E45" s="62" t="n"/>
-      <c r="F45" s="62" t="n"/>
-      <c r="G45" s="62" t="n"/>
-      <c r="H45" s="62" t="n"/>
+      <c r="A45" s="54" t="n"/>
+      <c r="B45" s="54" t="n"/>
+      <c r="C45" s="54" t="n"/>
+      <c r="D45" s="55" t="inlineStr">
+        <is>
+          <t>Data: 16/04/2026</t>
+        </is>
+      </c>
+      <c r="E45" s="54" t="n"/>
+      <c r="F45" s="54" t="n"/>
+      <c r="G45" s="54" t="n"/>
+      <c r="H45" s="54" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="19" t="inlineStr">
+      <c r="A46" s="26" t="inlineStr">
         <is>
           <t>_____________________________________</t>
         </is>
@@ -1766,7 +1740,7 @@
     <row r="47"/>
     <row r="48"/>
     <row r="49">
-      <c r="A49" s="26" t="inlineStr">
+      <c r="A49" s="28" t="inlineStr">
         <is>
           <t>Responsável pela Análise</t>
         </is>
@@ -1776,13 +1750,13 @@
   <mergeCells count="50">
     <mergeCell ref="A30:E30"/>
     <mergeCell ref="A34:E34"/>
+    <mergeCell ref="G12:H12"/>
     <mergeCell ref="D13:F13"/>
-    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="A39:H39"/>
     <mergeCell ref="F5:H5"/>
     <mergeCell ref="A24:E24"/>
+    <mergeCell ref="G2:H2"/>
     <mergeCell ref="A15:H15"/>
-    <mergeCell ref="G2:H2"/>
-    <mergeCell ref="A39:H39"/>
     <mergeCell ref="C9:E9"/>
     <mergeCell ref="A49:H49"/>
     <mergeCell ref="A12:C12"/>
@@ -1817,10 +1791,10 @@
     <mergeCell ref="A29:E29"/>
     <mergeCell ref="A20:E20"/>
     <mergeCell ref="C5:E5"/>
+    <mergeCell ref="A38:H38"/>
+    <mergeCell ref="A28:E28"/>
     <mergeCell ref="G1:H1"/>
     <mergeCell ref="C1:F3"/>
-    <mergeCell ref="A38:H38"/>
-    <mergeCell ref="A28:E28"/>
     <mergeCell ref="A19:E19"/>
     <mergeCell ref="A31:E31"/>
     <mergeCell ref="C10:E10"/>

</xml_diff>

<commit_message>
inclusão da classe instrumento TRANSMISSOR DE TEMPERATURA (ORIGEM)
</commit_message>
<xml_diff>
--- a/TemplateAC_ORIGEM.xlsx
+++ b/TemplateAC_ORIGEM.xlsx
@@ -372,7 +372,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -478,6 +478,33 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -989,25 +1016,25 @@
     <row r="6" ht="34.5" customHeight="1" s="23">
       <c r="A6" s="34" t="inlineStr">
         <is>
-          <t>FT-C-624005-02</t>
+          <t>PDIT-1900001A-01</t>
         </is>
       </c>
       <c r="B6" s="15" t="n"/>
       <c r="C6" s="34" t="inlineStr">
         <is>
-          <t>loc</t>
+          <t>teste</t>
         </is>
       </c>
       <c r="D6" s="14" t="n"/>
       <c r="E6" s="15" t="n"/>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>SAP: sap</t>
+          <t>SAP: teste</t>
         </is>
       </c>
       <c r="G6" s="34" t="inlineStr">
         <is>
-          <t>CE: nac</t>
+          <t>CE: teste</t>
         </is>
       </c>
       <c r="H6" s="15" t="n"/>
@@ -1095,14 +1122,14 @@
     <row r="13">
       <c r="A13" s="34" t="inlineStr">
         <is>
-          <t>26-ODS-0638-PRE-040</t>
+          <t>26-ODS-0638-PRE-043</t>
         </is>
       </c>
       <c r="B13" s="14" t="n"/>
       <c r="C13" s="15" t="n"/>
       <c r="D13" s="16" t="inlineStr">
         <is>
-          <t>09/04/2026</t>
+          <t>16/04/2026</t>
         </is>
       </c>
       <c r="E13" s="17" t="n"/>
@@ -1717,18 +1744,18 @@
       <c r="H43" s="33" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="54" t="n"/>
-      <c r="B45" s="54" t="n"/>
-      <c r="C45" s="54" t="n"/>
-      <c r="D45" s="55" t="inlineStr">
-        <is>
-          <t>Data: 16/04/2026</t>
-        </is>
-      </c>
-      <c r="E45" s="54" t="n"/>
-      <c r="F45" s="54" t="n"/>
-      <c r="G45" s="54" t="n"/>
-      <c r="H45" s="54" t="n"/>
+      <c r="A45" s="63" t="n"/>
+      <c r="B45" s="63" t="n"/>
+      <c r="C45" s="63" t="n"/>
+      <c r="D45" s="64" t="inlineStr">
+        <is>
+          <t>Data: 24/04/2026</t>
+        </is>
+      </c>
+      <c r="E45" s="63" t="n"/>
+      <c r="F45" s="63" t="n"/>
+      <c r="G45" s="63" t="n"/>
+      <c r="H45" s="63" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="26" t="inlineStr">

</xml_diff>

<commit_message>
ajuste nome da AC origem por n° da ac
</commit_message>
<xml_diff>
--- a/TemplateAC_ORIGEM.xlsx
+++ b/TemplateAC_ORIGEM.xlsx
@@ -372,7 +372,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="68">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -478,6 +478,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -1016,25 +1025,25 @@
     <row r="6" ht="34.5" customHeight="1" s="23">
       <c r="A6" s="34" t="inlineStr">
         <is>
-          <t>PDIT-1900001A-01</t>
+          <t>TT-1900001A-01</t>
         </is>
       </c>
       <c r="B6" s="15" t="n"/>
       <c r="C6" s="34" t="inlineStr">
         <is>
-          <t>teste</t>
+          <t>loc</t>
         </is>
       </c>
       <c r="D6" s="14" t="n"/>
       <c r="E6" s="15" t="n"/>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>SAP: teste</t>
+          <t>SAP: sap</t>
         </is>
       </c>
       <c r="G6" s="34" t="inlineStr">
         <is>
-          <t>CE: teste</t>
+          <t>CE: 123456</t>
         </is>
       </c>
       <c r="H6" s="15" t="n"/>
@@ -1076,7 +1085,7 @@
       <c r="B9" s="25" t="n"/>
       <c r="C9" s="27" t="inlineStr">
         <is>
-          <t>[ ✔ ] Transmissor de pressão diferencial (PDT)</t>
+          <t>[ ] Transmissor de pressão diferencial (PDT)</t>
         </is>
       </c>
       <c r="E9" s="25" t="n"/>
@@ -1088,7 +1097,7 @@
       <c r="B10" s="33" t="n"/>
       <c r="C10" s="47" t="inlineStr">
         <is>
-          <t>[ ] Transmissor de temperatura (TT)</t>
+          <t>[ ✔ ] Transmissor de temperatura (TT)</t>
         </is>
       </c>
       <c r="D10" s="37" t="n"/>
@@ -1122,7 +1131,7 @@
     <row r="13">
       <c r="A13" s="34" t="inlineStr">
         <is>
-          <t>26-ODS-0638-PRE-043</t>
+          <t>26-ODS-0638-TEM-024</t>
         </is>
       </c>
       <c r="B13" s="14" t="n"/>
@@ -1744,18 +1753,18 @@
       <c r="H43" s="33" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="63" t="n"/>
-      <c r="B45" s="63" t="n"/>
-      <c r="C45" s="63" t="n"/>
-      <c r="D45" s="64" t="inlineStr">
+      <c r="A45" s="66" t="n"/>
+      <c r="B45" s="66" t="n"/>
+      <c r="C45" s="66" t="n"/>
+      <c r="D45" s="67" t="inlineStr">
         <is>
           <t>Data: 24/04/2026</t>
         </is>
       </c>
-      <c r="E45" s="63" t="n"/>
-      <c r="F45" s="63" t="n"/>
-      <c r="G45" s="63" t="n"/>
-      <c r="H45" s="63" t="n"/>
+      <c r="E45" s="66" t="n"/>
+      <c r="F45" s="66" t="n"/>
+      <c r="G45" s="66" t="n"/>
+      <c r="H45" s="66" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="26" t="inlineStr">

</xml_diff>

<commit_message>
ajuste xml Transmissor de temperatura - origem
</commit_message>
<xml_diff>
--- a/TemplateAC_ORIGEM.xlsx
+++ b/TemplateAC_ORIGEM.xlsx
@@ -372,7 +372,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="78">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -478,6 +478,36 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -1025,7 +1055,7 @@
     <row r="6" ht="34.5" customHeight="1" s="23">
       <c r="A6" s="34" t="inlineStr">
         <is>
-          <t>TT-1900001A-01</t>
+          <t>TT-C-624005-02</t>
         </is>
       </c>
       <c r="B6" s="15" t="n"/>
@@ -1038,7 +1068,7 @@
       <c r="E6" s="15" t="n"/>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>SAP: sap</t>
+          <t>SAP: asda</t>
         </is>
       </c>
       <c r="G6" s="34" t="inlineStr">
@@ -1131,14 +1161,14 @@
     <row r="13">
       <c r="A13" s="34" t="inlineStr">
         <is>
-          <t>26-ODS-0638-TEM-024</t>
+          <t>26-ODS-0638-TEM-021</t>
         </is>
       </c>
       <c r="B13" s="14" t="n"/>
       <c r="C13" s="15" t="n"/>
       <c r="D13" s="16" t="inlineStr">
         <is>
-          <t>16/04/2026</t>
+          <t>09/04/2026</t>
         </is>
       </c>
       <c r="E13" s="17" t="n"/>
@@ -1733,7 +1763,17 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="35" t="inlineStr"/>
+      <c r="A42" s="35" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t xml:space="preserve">Novo NS alterado no computador de vazão / XML / SFP
+</t>
+          </r>
+        </is>
+      </c>
       <c r="B42" s="36" t="n"/>
       <c r="C42" s="36" t="n"/>
       <c r="D42" s="36" t="n"/>
@@ -1753,18 +1793,18 @@
       <c r="H43" s="33" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="66" t="n"/>
-      <c r="B45" s="66" t="n"/>
-      <c r="C45" s="66" t="n"/>
-      <c r="D45" s="67" t="inlineStr">
-        <is>
-          <t>Data: 24/04/2026</t>
-        </is>
-      </c>
-      <c r="E45" s="66" t="n"/>
-      <c r="F45" s="66" t="n"/>
-      <c r="G45" s="66" t="n"/>
-      <c r="H45" s="66" t="n"/>
+      <c r="A45" s="76" t="n"/>
+      <c r="B45" s="76" t="n"/>
+      <c r="C45" s="76" t="n"/>
+      <c r="D45" s="77" t="inlineStr">
+        <is>
+          <t>Data: 20/04/2026</t>
+        </is>
+      </c>
+      <c r="E45" s="76" t="n"/>
+      <c r="F45" s="76" t="n"/>
+      <c r="G45" s="76" t="n"/>
+      <c r="H45" s="76" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="26" t="inlineStr">

</xml_diff>

<commit_message>
validação do xsd e geração de log
</commit_message>
<xml_diff>
--- a/TemplateAC_ORIGEM.xlsx
+++ b/TemplateAC_ORIGEM.xlsx
@@ -372,7 +372,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="78">
+  <cellXfs count="84">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -478,6 +478,24 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -1068,12 +1086,12 @@
       <c r="E6" s="15" t="n"/>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>SAP: asda</t>
+          <t>SAP: sap</t>
         </is>
       </c>
       <c r="G6" s="34" t="inlineStr">
         <is>
-          <t>CE: 123456</t>
+          <t>CE: 6</t>
         </is>
       </c>
       <c r="H6" s="15" t="n"/>
@@ -1763,17 +1781,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="35" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <b val="1"/>
-            </rPr>
-            <t xml:space="preserve">Novo NS alterado no computador de vazão / XML / SFP
-</t>
-          </r>
-        </is>
-      </c>
+      <c r="A42" s="35" t="inlineStr"/>
       <c r="B42" s="36" t="n"/>
       <c r="C42" s="36" t="n"/>
       <c r="D42" s="36" t="n"/>
@@ -1793,18 +1801,18 @@
       <c r="H43" s="33" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="76" t="n"/>
-      <c r="B45" s="76" t="n"/>
-      <c r="C45" s="76" t="n"/>
-      <c r="D45" s="77" t="inlineStr">
+      <c r="A45" s="82" t="n"/>
+      <c r="B45" s="82" t="n"/>
+      <c r="C45" s="82" t="n"/>
+      <c r="D45" s="83" t="inlineStr">
         <is>
           <t>Data: 20/04/2026</t>
         </is>
       </c>
-      <c r="E45" s="76" t="n"/>
-      <c r="F45" s="76" t="n"/>
-      <c r="G45" s="76" t="n"/>
-      <c r="H45" s="76" t="n"/>
+      <c r="E45" s="82" t="n"/>
+      <c r="F45" s="82" t="n"/>
+      <c r="G45" s="82" t="n"/>
+      <c r="H45" s="82" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="26" t="inlineStr">

</xml_diff>

<commit_message>
ajuste tabela as found as left instrumentos de pressão - xml petro
</commit_message>
<xml_diff>
--- a/TemplateAC_ORIGEM.xlsx
+++ b/TemplateAC_ORIGEM.xlsx
@@ -372,7 +372,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="87">
+  <cellXfs count="89">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -478,6 +478,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -1082,25 +1088,25 @@
     <row r="6" ht="34.5" customHeight="1" s="23">
       <c r="A6" s="34" t="inlineStr">
         <is>
-          <t>TE-1900001A-02</t>
+          <t>UT-SG-122101-01</t>
         </is>
       </c>
       <c r="B6" s="15" t="n"/>
       <c r="C6" s="34" t="inlineStr">
         <is>
-          <t>TESTE</t>
+          <t>teste</t>
         </is>
       </c>
       <c r="D6" s="14" t="n"/>
       <c r="E6" s="15" t="n"/>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>SAP: TESTE</t>
+          <t>SAP: teste</t>
         </is>
       </c>
       <c r="G6" s="34" t="inlineStr">
         <is>
-          <t>CE: TESTE</t>
+          <t>CE: teste</t>
         </is>
       </c>
       <c r="H6" s="15" t="n"/>
@@ -1131,7 +1137,7 @@
       <c r="E8" s="30" t="n"/>
       <c r="F8" s="34" t="inlineStr">
         <is>
-          <t>[ ✔ ] Termorresistência (TE)</t>
+          <t>[ ] Termorresistência (TE)</t>
         </is>
       </c>
       <c r="G8" s="36" t="n"/>
@@ -1142,7 +1148,7 @@
       <c r="B9" s="25" t="n"/>
       <c r="C9" s="27" t="inlineStr">
         <is>
-          <t>[ ] Transmissor de pressão diferencial (PDT)</t>
+          <t>[ ✔ ] Transmissor de pressão diferencial (PDT)</t>
         </is>
       </c>
       <c r="E9" s="25" t="n"/>
@@ -1188,14 +1194,14 @@
     <row r="13">
       <c r="A13" s="34" t="inlineStr">
         <is>
-          <t>26-ODS-0638-TEM-235</t>
+          <t>26-ODS-0638-PRE-444</t>
         </is>
       </c>
       <c r="B13" s="14" t="n"/>
       <c r="C13" s="15" t="n"/>
       <c r="D13" s="16" t="inlineStr">
         <is>
-          <t>28/04/2026</t>
+          <t>09/04/2026</t>
         </is>
       </c>
       <c r="E13" s="17" t="n"/>
@@ -1730,7 +1736,7 @@
       <c r="E35" s="15" t="n"/>
       <c r="F35" s="10" t="inlineStr">
         <is>
-          <t>○</t>
+          <t>◉</t>
         </is>
       </c>
       <c r="G35" s="10" t="inlineStr">
@@ -1740,7 +1746,7 @@
       </c>
       <c r="H35" s="10" t="inlineStr">
         <is>
-          <t>◉</t>
+          <t>○</t>
         </is>
       </c>
     </row>
@@ -1810,18 +1816,18 @@
       <c r="H43" s="33" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="85" t="n"/>
-      <c r="B45" s="85" t="n"/>
-      <c r="C45" s="85" t="n"/>
-      <c r="D45" s="86" t="inlineStr">
-        <is>
-          <t>Data: 30/04/2026</t>
-        </is>
-      </c>
-      <c r="E45" s="85" t="n"/>
-      <c r="F45" s="85" t="n"/>
-      <c r="G45" s="85" t="n"/>
-      <c r="H45" s="85" t="n"/>
+      <c r="A45" s="87" t="n"/>
+      <c r="B45" s="87" t="n"/>
+      <c r="C45" s="87" t="n"/>
+      <c r="D45" s="88" t="inlineStr">
+        <is>
+          <t>Data: 15/04/2026</t>
+        </is>
+      </c>
+      <c r="E45" s="87" t="n"/>
+      <c r="F45" s="87" t="n"/>
+      <c r="G45" s="87" t="n"/>
+      <c r="H45" s="87" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="26" t="inlineStr">

</xml_diff>

<commit_message>
ajuste parser NS sec e placa
</commit_message>
<xml_diff>
--- a/TemplateAC_ORIGEM.xlsx
+++ b/TemplateAC_ORIGEM.xlsx
@@ -372,7 +372,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="89">
+  <cellXfs count="95">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -478,6 +478,24 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -1088,7 +1106,7 @@
     <row r="6" ht="34.5" customHeight="1" s="23">
       <c r="A6" s="34" t="inlineStr">
         <is>
-          <t>UT-SG-122101-01</t>
+          <t>PDIT-1900002A-02</t>
         </is>
       </c>
       <c r="B6" s="15" t="n"/>
@@ -1194,14 +1212,14 @@
     <row r="13">
       <c r="A13" s="34" t="inlineStr">
         <is>
-          <t>26-ODS-0638-PRE-444</t>
+          <t>26-ODS-0638-PRE-452</t>
         </is>
       </c>
       <c r="B13" s="14" t="n"/>
       <c r="C13" s="15" t="n"/>
       <c r="D13" s="16" t="inlineStr">
         <is>
-          <t>09/04/2026</t>
+          <t>27/04/2026</t>
         </is>
       </c>
       <c r="E13" s="17" t="n"/>
@@ -1736,17 +1754,17 @@
       <c r="E35" s="15" t="n"/>
       <c r="F35" s="10" t="inlineStr">
         <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="G35" s="10" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H35" s="10" t="inlineStr">
+        <is>
           <t>◉</t>
-        </is>
-      </c>
-      <c r="G35" s="10" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="H35" s="10" t="inlineStr">
-        <is>
-          <t>○</t>
         </is>
       </c>
     </row>
@@ -1816,18 +1834,18 @@
       <c r="H43" s="33" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="87" t="n"/>
-      <c r="B45" s="87" t="n"/>
-      <c r="C45" s="87" t="n"/>
-      <c r="D45" s="88" t="inlineStr">
-        <is>
-          <t>Data: 15/04/2026</t>
-        </is>
-      </c>
-      <c r="E45" s="87" t="n"/>
-      <c r="F45" s="87" t="n"/>
-      <c r="G45" s="87" t="n"/>
-      <c r="H45" s="87" t="n"/>
+      <c r="A45" s="93" t="n"/>
+      <c r="B45" s="93" t="n"/>
+      <c r="C45" s="93" t="n"/>
+      <c r="D45" s="94" t="inlineStr">
+        <is>
+          <t>Data: 30/04/2026</t>
+        </is>
+      </c>
+      <c r="E45" s="93" t="n"/>
+      <c r="F45" s="93" t="n"/>
+      <c r="G45" s="93" t="n"/>
+      <c r="H45" s="93" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="26" t="inlineStr">

</xml_diff>

<commit_message>
validação de xml de trecho reto de gás com porta placas
</commit_message>
<xml_diff>
--- a/TemplateAC_ORIGEM.xlsx
+++ b/TemplateAC_ORIGEM.xlsx
@@ -372,7 +372,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="95">
+  <cellXfs count="96">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -478,6 +478,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -1106,25 +1109,25 @@
     <row r="6" ht="34.5" customHeight="1" s="23">
       <c r="A6" s="34" t="inlineStr">
         <is>
-          <t>PDIT-1900002A-02</t>
+          <t>UT-SG-122101-01</t>
         </is>
       </c>
       <c r="B6" s="15" t="n"/>
       <c r="C6" s="34" t="inlineStr">
         <is>
-          <t>teste</t>
+          <t>TESTE</t>
         </is>
       </c>
       <c r="D6" s="14" t="n"/>
       <c r="E6" s="15" t="n"/>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>SAP: teste</t>
+          <t>SAP: TESTE</t>
         </is>
       </c>
       <c r="G6" s="34" t="inlineStr">
         <is>
-          <t>CE: teste</t>
+          <t>CE: TESTE</t>
         </is>
       </c>
       <c r="H6" s="15" t="n"/>
@@ -1212,14 +1215,14 @@
     <row r="13">
       <c r="A13" s="34" t="inlineStr">
         <is>
-          <t>26-ODS-0638-PRE-452</t>
+          <t>26-ODS-0638-PRE-444</t>
         </is>
       </c>
       <c r="B13" s="14" t="n"/>
       <c r="C13" s="15" t="n"/>
       <c r="D13" s="16" t="inlineStr">
         <is>
-          <t>27/04/2026</t>
+          <t>09/04/2026</t>
         </is>
       </c>
       <c r="E13" s="17" t="n"/>
@@ -1754,7 +1757,7 @@
       <c r="E35" s="15" t="n"/>
       <c r="F35" s="10" t="inlineStr">
         <is>
-          <t>○</t>
+          <t>◉</t>
         </is>
       </c>
       <c r="G35" s="10" t="inlineStr">
@@ -1764,7 +1767,7 @@
       </c>
       <c r="H35" s="10" t="inlineStr">
         <is>
-          <t>◉</t>
+          <t>○</t>
         </is>
       </c>
     </row>
@@ -1834,18 +1837,18 @@
       <c r="H43" s="33" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="93" t="n"/>
-      <c r="B45" s="93" t="n"/>
-      <c r="C45" s="93" t="n"/>
-      <c r="D45" s="94" t="inlineStr">
-        <is>
-          <t>Data: 30/04/2026</t>
-        </is>
-      </c>
-      <c r="E45" s="93" t="n"/>
-      <c r="F45" s="93" t="n"/>
-      <c r="G45" s="93" t="n"/>
-      <c r="H45" s="93" t="n"/>
+      <c r="A45" s="94" t="n"/>
+      <c r="B45" s="94" t="n"/>
+      <c r="C45" s="94" t="n"/>
+      <c r="D45" s="95" t="inlineStr">
+        <is>
+          <t>Data: 15/04/2026</t>
+        </is>
+      </c>
+      <c r="E45" s="94" t="n"/>
+      <c r="F45" s="94" t="n"/>
+      <c r="G45" s="94" t="n"/>
+      <c r="H45" s="94" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="26" t="inlineStr">

</xml_diff>

<commit_message>
import e export bd via xlsx
</commit_message>
<xml_diff>
--- a/TemplateAC_ORIGEM.xlsx
+++ b/TemplateAC_ORIGEM.xlsx
@@ -372,7 +372,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="96">
+  <cellXfs count="100">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -478,6 +478,18 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -1109,25 +1121,25 @@
     <row r="6" ht="34.5" customHeight="1" s="23">
       <c r="A6" s="34" t="inlineStr">
         <is>
-          <t>UT-SG-122101-01</t>
+          <t>TIT-1900002A-01</t>
         </is>
       </c>
       <c r="B6" s="15" t="n"/>
       <c r="C6" s="34" t="inlineStr">
         <is>
-          <t>TESTE</t>
+          <t>teste</t>
         </is>
       </c>
       <c r="D6" s="14" t="n"/>
       <c r="E6" s="15" t="n"/>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>SAP: TESTE</t>
+          <t>SAP: teste</t>
         </is>
       </c>
       <c r="G6" s="34" t="inlineStr">
         <is>
-          <t>CE: TESTE</t>
+          <t>CE: teste</t>
         </is>
       </c>
       <c r="H6" s="15" t="n"/>
@@ -1169,7 +1181,7 @@
       <c r="B9" s="25" t="n"/>
       <c r="C9" s="27" t="inlineStr">
         <is>
-          <t>[ ✔ ] Transmissor de pressão diferencial (PDT)</t>
+          <t>[ ] Transmissor de pressão diferencial (PDT)</t>
         </is>
       </c>
       <c r="E9" s="25" t="n"/>
@@ -1181,7 +1193,7 @@
       <c r="B10" s="33" t="n"/>
       <c r="C10" s="47" t="inlineStr">
         <is>
-          <t>[ ] Transmissor de temperatura (TT)</t>
+          <t>[ ✔ ] Transmissor de temperatura (TT)</t>
         </is>
       </c>
       <c r="D10" s="37" t="n"/>
@@ -1215,14 +1227,14 @@
     <row r="13">
       <c r="A13" s="34" t="inlineStr">
         <is>
-          <t>26-ODS-0638-PRE-444</t>
+          <t>26-ODS-0638-TEM-230</t>
         </is>
       </c>
       <c r="B13" s="14" t="n"/>
       <c r="C13" s="15" t="n"/>
       <c r="D13" s="16" t="inlineStr">
         <is>
-          <t>09/04/2026</t>
+          <t>23/04/2026</t>
         </is>
       </c>
       <c r="E13" s="17" t="n"/>
@@ -1757,17 +1769,17 @@
       <c r="E35" s="15" t="n"/>
       <c r="F35" s="10" t="inlineStr">
         <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="G35" s="10" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="H35" s="10" t="inlineStr">
+        <is>
           <t>◉</t>
-        </is>
-      </c>
-      <c r="G35" s="10" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="H35" s="10" t="inlineStr">
-        <is>
-          <t>○</t>
         </is>
       </c>
     </row>
@@ -1837,18 +1849,18 @@
       <c r="H43" s="33" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="94" t="n"/>
-      <c r="B45" s="94" t="n"/>
-      <c r="C45" s="94" t="n"/>
-      <c r="D45" s="95" t="inlineStr">
-        <is>
-          <t>Data: 15/04/2026</t>
-        </is>
-      </c>
-      <c r="E45" s="94" t="n"/>
-      <c r="F45" s="94" t="n"/>
-      <c r="G45" s="94" t="n"/>
-      <c r="H45" s="94" t="n"/>
+      <c r="A45" s="98" t="n"/>
+      <c r="B45" s="98" t="n"/>
+      <c r="C45" s="98" t="n"/>
+      <c r="D45" s="99" t="inlineStr">
+        <is>
+          <t>Data: 29/04/2026</t>
+        </is>
+      </c>
+      <c r="E45" s="98" t="n"/>
+      <c r="F45" s="98" t="n"/>
+      <c r="G45" s="98" t="n"/>
+      <c r="H45" s="98" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="26" t="inlineStr">

</xml_diff>

<commit_message>
ajuste xml CI - formatação caractere inválida
</commit_message>
<xml_diff>
--- a/TemplateAC_ORIGEM.xlsx
+++ b/TemplateAC_ORIGEM.xlsx
@@ -372,7 +372,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="100">
+  <cellXfs count="101">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -478,6 +478,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -1121,7 +1124,7 @@
     <row r="6" ht="34.5" customHeight="1" s="23">
       <c r="A6" s="34" t="inlineStr">
         <is>
-          <t>TIT-1900002A-01</t>
+          <t>TT-SG-122103-01A</t>
         </is>
       </c>
       <c r="B6" s="15" t="n"/>
@@ -1170,7 +1173,7 @@
       <c r="E8" s="30" t="n"/>
       <c r="F8" s="34" t="inlineStr">
         <is>
-          <t>[ ] Termorresistência (TE)</t>
+          <t>[ ✔ ] Termorresistência (TE)</t>
         </is>
       </c>
       <c r="G8" s="36" t="n"/>
@@ -1227,14 +1230,14 @@
     <row r="13">
       <c r="A13" s="34" t="inlineStr">
         <is>
-          <t>26-ODS-0638-TEM-230</t>
+          <t>26-ODS-0638-TEM-112</t>
         </is>
       </c>
       <c r="B13" s="14" t="n"/>
       <c r="C13" s="15" t="n"/>
       <c r="D13" s="16" t="inlineStr">
         <is>
-          <t>23/04/2026</t>
+          <t>06/05/2026</t>
         </is>
       </c>
       <c r="E13" s="17" t="n"/>
@@ -1849,18 +1852,18 @@
       <c r="H43" s="33" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="98" t="n"/>
-      <c r="B45" s="98" t="n"/>
-      <c r="C45" s="98" t="n"/>
-      <c r="D45" s="99" t="inlineStr">
-        <is>
-          <t>Data: 29/04/2026</t>
-        </is>
-      </c>
-      <c r="E45" s="98" t="n"/>
-      <c r="F45" s="98" t="n"/>
-      <c r="G45" s="98" t="n"/>
-      <c r="H45" s="98" t="n"/>
+      <c r="A45" s="99" t="n"/>
+      <c r="B45" s="99" t="n"/>
+      <c r="C45" s="99" t="n"/>
+      <c r="D45" s="100" t="inlineStr">
+        <is>
+          <t>Data: 18/05/2026</t>
+        </is>
+      </c>
+      <c r="E45" s="99" t="n"/>
+      <c r="F45" s="99" t="n"/>
+      <c r="G45" s="99" t="n"/>
+      <c r="H45" s="99" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="26" t="inlineStr">

</xml_diff>

<commit_message>
ajuste de certificado de placa
</commit_message>
<xml_diff>
--- a/TemplateAC_ORIGEM.xlsx
+++ b/TemplateAC_ORIGEM.xlsx
@@ -372,7 +372,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="101">
+  <cellXfs count="102">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -478,6 +478,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -1124,25 +1127,25 @@
     <row r="6" ht="34.5" customHeight="1" s="23">
       <c r="A6" s="34" t="inlineStr">
         <is>
-          <t>TT-SG-122103-01A</t>
+          <t>TIT-1900003</t>
         </is>
       </c>
       <c r="B6" s="15" t="n"/>
       <c r="C6" s="34" t="inlineStr">
         <is>
-          <t>teste</t>
+          <t>tes</t>
         </is>
       </c>
       <c r="D6" s="14" t="n"/>
       <c r="E6" s="15" t="n"/>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>SAP: teste</t>
+          <t>SAP: texs</t>
         </is>
       </c>
       <c r="G6" s="34" t="inlineStr">
         <is>
-          <t>CE: teste</t>
+          <t>CE: tes</t>
         </is>
       </c>
       <c r="H6" s="15" t="n"/>
@@ -1173,7 +1176,7 @@
       <c r="E8" s="30" t="n"/>
       <c r="F8" s="34" t="inlineStr">
         <is>
-          <t>[ ✔ ] Termorresistência (TE)</t>
+          <t>[ ] Termorresistência (TE)</t>
         </is>
       </c>
       <c r="G8" s="36" t="n"/>
@@ -1230,14 +1233,14 @@
     <row r="13">
       <c r="A13" s="34" t="inlineStr">
         <is>
-          <t>26-ODS-0638-TEM-112</t>
+          <t>26-ODS-0638-TEM-246</t>
         </is>
       </c>
       <c r="B13" s="14" t="n"/>
       <c r="C13" s="15" t="n"/>
       <c r="D13" s="16" t="inlineStr">
         <is>
-          <t>06/05/2026</t>
+          <t>22/05/2026</t>
         </is>
       </c>
       <c r="E13" s="17" t="n"/>
@@ -1852,18 +1855,18 @@
       <c r="H43" s="33" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="99" t="n"/>
-      <c r="B45" s="99" t="n"/>
-      <c r="C45" s="99" t="n"/>
-      <c r="D45" s="100" t="inlineStr">
-        <is>
-          <t>Data: 18/05/2026</t>
-        </is>
-      </c>
-      <c r="E45" s="99" t="n"/>
-      <c r="F45" s="99" t="n"/>
-      <c r="G45" s="99" t="n"/>
-      <c r="H45" s="99" t="n"/>
+      <c r="A45" s="100" t="n"/>
+      <c r="B45" s="100" t="n"/>
+      <c r="C45" s="100" t="n"/>
+      <c r="D45" s="101" t="inlineStr">
+        <is>
+          <t>Data: 29/05/2026</t>
+        </is>
+      </c>
+      <c r="E45" s="100" t="n"/>
+      <c r="F45" s="100" t="n"/>
+      <c r="G45" s="100" t="n"/>
+      <c r="H45" s="100" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="26" t="inlineStr">

</xml_diff>